<commit_message>
firebase tiempo real funcionando
</commit_message>
<xml_diff>
--- a/Invitados.xlsx
+++ b/Invitados.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ipera\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ipera\Desktop\Ceremonia-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{667B3F52-11EC-4423-9EDF-DA801C9983CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD6CC94-E404-44E6-B55D-895B0CA75B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3424,10 +3424,10 @@
       <c r="P1" s="1" t="s">
         <v>946</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="1" t="s">
         <v>947</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="1" t="s">
         <v>948</v>
       </c>
     </row>
@@ -3460,6 +3460,8 @@
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
@@ -3490,6 +3492,8 @@
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
@@ -3520,6 +3524,8 @@
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
@@ -3552,6 +3558,8 @@
       </c>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
@@ -3584,6 +3592,8 @@
       </c>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
@@ -3614,6 +3624,8 @@
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
+      <c r="R7" s="4"/>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
@@ -3644,6 +3656,8 @@
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
@@ -3674,6 +3688,8 @@
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
@@ -3704,6 +3720,8 @@
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
@@ -3734,6 +3752,8 @@
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
       <c r="P11" s="4"/>
+      <c r="Q11" s="4"/>
+      <c r="R11" s="4"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
@@ -3764,6 +3784,8 @@
       <c r="N12" s="4"/>
       <c r="O12" s="4"/>
       <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
@@ -3794,6 +3816,8 @@
       <c r="N13" s="4"/>
       <c r="O13" s="4"/>
       <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
+      <c r="R13" s="4"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
@@ -3824,6 +3848,8 @@
       <c r="N14" s="4"/>
       <c r="O14" s="4"/>
       <c r="P14" s="4"/>
+      <c r="Q14" s="4"/>
+      <c r="R14" s="4"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
@@ -3854,6 +3880,8 @@
       <c r="N15" s="4"/>
       <c r="O15" s="4"/>
       <c r="P15" s="4"/>
+      <c r="Q15" s="4"/>
+      <c r="R15" s="4"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
@@ -3884,8 +3912,10 @@
       <c r="N16" s="4"/>
       <c r="O16" s="4"/>
       <c r="P16" s="4"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q16" s="4"/>
+      <c r="R16" s="4"/>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -3914,8 +3944,10 @@
       <c r="N17" s="4"/>
       <c r="O17" s="4"/>
       <c r="P17" s="4"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q17" s="4"/>
+      <c r="R17" s="4"/>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -3944,8 +3976,10 @@
       <c r="N18" s="4"/>
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q18" s="4"/>
+      <c r="R18" s="4"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -3976,8 +4010,10 @@
       </c>
       <c r="O19" s="4"/>
       <c r="P19" s="4"/>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q19" s="4"/>
+      <c r="R19" s="4"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -4006,8 +4042,10 @@
       <c r="N20" s="4"/>
       <c r="O20" s="4"/>
       <c r="P20" s="4"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q20" s="4"/>
+      <c r="R20" s="4"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -4036,8 +4074,10 @@
       <c r="N21" s="4"/>
       <c r="O21" s="4"/>
       <c r="P21" s="4"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q21" s="4"/>
+      <c r="R21" s="4"/>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A22" s="4">
         <v>21</v>
       </c>
@@ -4066,8 +4106,10 @@
       <c r="N22" s="4"/>
       <c r="O22" s="4"/>
       <c r="P22" s="4"/>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q22" s="4"/>
+      <c r="R22" s="4"/>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A23" s="4">
         <v>22</v>
       </c>
@@ -4096,8 +4138,10 @@
       <c r="N23" s="4"/>
       <c r="O23" s="4"/>
       <c r="P23" s="4"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q23" s="4"/>
+      <c r="R23" s="4"/>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A24" s="4">
         <v>23</v>
       </c>
@@ -4126,8 +4170,10 @@
       <c r="N24" s="4"/>
       <c r="O24" s="4"/>
       <c r="P24" s="4"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q24" s="4"/>
+      <c r="R24" s="4"/>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A25" s="4">
         <v>24</v>
       </c>
@@ -4156,8 +4202,10 @@
       </c>
       <c r="O25" s="4"/>
       <c r="P25" s="4"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q25" s="4"/>
+      <c r="R25" s="4"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>25</v>
       </c>
@@ -4202,8 +4250,10 @@
       <c r="P26" s="5">
         <v>22</v>
       </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q26" s="5"/>
+      <c r="R26" s="5"/>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>26</v>
       </c>
@@ -4248,8 +4298,10 @@
       <c r="P27" s="5">
         <v>20</v>
       </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q27" s="5"/>
+      <c r="R27" s="5"/>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>27</v>
       </c>
@@ -4294,8 +4346,10 @@
       <c r="P28" s="5">
         <v>19</v>
       </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q28" s="5"/>
+      <c r="R28" s="5"/>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>28</v>
       </c>
@@ -4340,8 +4394,10 @@
       <c r="P29" s="5">
         <v>19</v>
       </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q29" s="5"/>
+      <c r="R29" s="5"/>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>29</v>
       </c>
@@ -4386,8 +4442,10 @@
       <c r="P30" s="5">
         <v>19</v>
       </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q30" s="5"/>
+      <c r="R30" s="5"/>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>30</v>
       </c>
@@ -4432,8 +4490,10 @@
       <c r="P31" s="5">
         <v>19</v>
       </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q31" s="5"/>
+      <c r="R31" s="5"/>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>31</v>
       </c>
@@ -4478,8 +4538,10 @@
       <c r="P32" s="5">
         <v>19</v>
       </c>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q32" s="5"/>
+      <c r="R32" s="5"/>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>32</v>
       </c>
@@ -4524,8 +4586,10 @@
       <c r="P33" s="5">
         <v>19</v>
       </c>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q33" s="5"/>
+      <c r="R33" s="5"/>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>33</v>
       </c>
@@ -4570,8 +4634,10 @@
       <c r="P34" s="5">
         <v>19</v>
       </c>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q34" s="5"/>
+      <c r="R34" s="5"/>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
         <v>34</v>
       </c>
@@ -4616,8 +4682,10 @@
       <c r="P35" s="5">
         <v>19</v>
       </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q35" s="5"/>
+      <c r="R35" s="5"/>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
         <v>35</v>
       </c>
@@ -4662,8 +4730,10 @@
       <c r="P36" s="5">
         <v>18</v>
       </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q36" s="5"/>
+      <c r="R36" s="5"/>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
         <v>36</v>
       </c>
@@ -4708,8 +4778,10 @@
       <c r="P37" s="5">
         <v>18</v>
       </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q37" s="5"/>
+      <c r="R37" s="5"/>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
         <v>37</v>
       </c>
@@ -4754,8 +4826,10 @@
       <c r="P38" s="5">
         <v>18</v>
       </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q38" s="5"/>
+      <c r="R38" s="5"/>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
         <v>38</v>
       </c>
@@ -4800,8 +4874,10 @@
       <c r="P39" s="5">
         <v>18</v>
       </c>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q39" s="5"/>
+      <c r="R39" s="5"/>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
         <v>39</v>
       </c>
@@ -4846,8 +4922,10 @@
       <c r="P40" s="5">
         <v>18</v>
       </c>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q40" s="5"/>
+      <c r="R40" s="5"/>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A41" s="15">
         <v>40</v>
       </c>
@@ -4886,8 +4964,10 @@
       <c r="P41" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q41" s="15"/>
+      <c r="R41" s="15"/>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A42" s="15">
         <v>41</v>
       </c>
@@ -4926,8 +5006,10 @@
       <c r="P42" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q42" s="15"/>
+      <c r="R42" s="15"/>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A43" s="15">
         <v>42</v>
       </c>
@@ -4966,8 +5048,10 @@
       <c r="P43" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q43" s="15"/>
+      <c r="R43" s="15"/>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A44" s="15">
         <v>43</v>
       </c>
@@ -5006,8 +5090,10 @@
       <c r="P44" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q44" s="15"/>
+      <c r="R44" s="15"/>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A45" s="15">
         <v>44</v>
       </c>
@@ -5046,8 +5132,10 @@
       <c r="P45" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q45" s="15"/>
+      <c r="R45" s="15"/>
+    </row>
+    <row r="46" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A46" s="15">
         <v>45</v>
       </c>
@@ -5086,8 +5174,10 @@
       <c r="P46" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q46" s="15"/>
+      <c r="R46" s="15"/>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A47" s="15">
         <v>46</v>
       </c>
@@ -5126,8 +5216,10 @@
       <c r="P47" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q47" s="15"/>
+      <c r="R47" s="15"/>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A48" s="15">
         <v>47</v>
       </c>
@@ -5166,8 +5258,10 @@
       <c r="P48" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q48" s="15"/>
+      <c r="R48" s="15"/>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A49" s="15">
         <v>48</v>
       </c>
@@ -5206,8 +5300,10 @@
       <c r="P49" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q49" s="15"/>
+      <c r="R49" s="15"/>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A50" s="15">
         <v>49</v>
       </c>
@@ -5246,8 +5342,10 @@
       <c r="P50" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q50" s="15"/>
+      <c r="R50" s="15"/>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A51" s="15">
         <v>50</v>
       </c>
@@ -5286,8 +5384,10 @@
       <c r="P51" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q51" s="15"/>
+      <c r="R51" s="15"/>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A52" s="15">
         <v>51</v>
       </c>
@@ -5328,8 +5428,10 @@
       <c r="P52" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q52" s="15"/>
+      <c r="R52" s="15"/>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A53" s="15">
         <v>52</v>
       </c>
@@ -5370,8 +5472,10 @@
       <c r="P53" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q53" s="15"/>
+      <c r="R53" s="15"/>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A54" s="15">
         <v>53</v>
       </c>
@@ -5412,8 +5516,10 @@
       <c r="P54" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q54" s="15"/>
+      <c r="R54" s="15"/>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A55" s="15">
         <v>54</v>
       </c>
@@ -5454,8 +5560,10 @@
       <c r="P55" s="15">
         <v>18</v>
       </c>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q55" s="15"/>
+      <c r="R55" s="15"/>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A56" s="5">
         <v>55</v>
       </c>
@@ -5498,8 +5606,10 @@
       <c r="P56" s="5">
         <v>17</v>
       </c>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q56" s="5"/>
+      <c r="R56" s="5"/>
+    </row>
+    <row r="57" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A57" s="15">
         <v>56</v>
       </c>
@@ -5538,8 +5648,10 @@
       <c r="P57" s="15">
         <v>17</v>
       </c>
-    </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q57" s="15"/>
+      <c r="R57" s="15"/>
+    </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A58" s="15">
         <v>57</v>
       </c>
@@ -5578,8 +5690,10 @@
       <c r="P58" s="15">
         <v>17</v>
       </c>
-    </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q58" s="15"/>
+      <c r="R58" s="15"/>
+    </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A59" s="15">
         <v>58</v>
       </c>
@@ -5618,8 +5732,10 @@
       <c r="P59" s="15">
         <v>17</v>
       </c>
-    </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q59" s="15"/>
+      <c r="R59" s="15"/>
+    </row>
+    <row r="60" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A60" s="15">
         <v>59</v>
       </c>
@@ -5658,8 +5774,10 @@
       <c r="P60" s="15">
         <v>17</v>
       </c>
-    </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q60" s="15"/>
+      <c r="R60" s="15"/>
+    </row>
+    <row r="61" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A61" s="15">
         <v>60</v>
       </c>
@@ -5698,8 +5816,10 @@
       <c r="P61" s="15">
         <v>17</v>
       </c>
-    </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q61" s="15"/>
+      <c r="R61" s="15"/>
+    </row>
+    <row r="62" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A62" s="15">
         <v>61</v>
       </c>
@@ -5740,8 +5860,10 @@
       <c r="P62" s="15">
         <v>17</v>
       </c>
-    </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q62" s="15"/>
+      <c r="R62" s="15"/>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A63" s="15">
         <v>62</v>
       </c>
@@ -5782,8 +5904,10 @@
       <c r="P63" s="15">
         <v>17</v>
       </c>
-    </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q63" s="15"/>
+      <c r="R63" s="15"/>
+    </row>
+    <row r="64" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A64" s="15">
         <v>63</v>
       </c>
@@ -5822,8 +5946,10 @@
       <c r="P64" s="15">
         <v>17</v>
       </c>
-    </row>
-    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+      <c r="Q64" s="15"/>
+      <c r="R64" s="15"/>
+    </row>
+    <row r="65" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="5">
         <v>44</v>
       </c>
@@ -5868,8 +5994,10 @@
       <c r="P65" s="5">
         <v>18</v>
       </c>
-    </row>
-    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+      <c r="Q65" s="5"/>
+      <c r="R65" s="5"/>
+    </row>
+    <row r="66" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5">
         <v>45</v>
       </c>
@@ -5914,8 +6042,10 @@
       <c r="P66" s="5">
         <v>18</v>
       </c>
-    </row>
-    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+      <c r="Q66" s="5"/>
+      <c r="R66" s="5"/>
+    </row>
+    <row r="67" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="5">
         <v>46</v>
       </c>
@@ -5960,8 +6090,10 @@
       <c r="P67" s="5">
         <v>18</v>
       </c>
-    </row>
-    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+      <c r="Q67" s="5"/>
+      <c r="R67" s="5"/>
+    </row>
+    <row r="68" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="5">
         <v>47</v>
       </c>
@@ -6006,8 +6138,10 @@
       <c r="P68" s="5">
         <v>18</v>
       </c>
-    </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q68" s="5"/>
+      <c r="R68" s="5"/>
+    </row>
+    <row r="69" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A69" s="5">
         <v>64</v>
       </c>
@@ -6050,8 +6184,10 @@
       <c r="P69" s="5">
         <v>17</v>
       </c>
-    </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q69" s="5"/>
+      <c r="R69" s="5"/>
+    </row>
+    <row r="70" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A70" s="15">
         <v>65</v>
       </c>
@@ -6090,8 +6226,10 @@
       <c r="P70" s="15">
         <v>17</v>
       </c>
-    </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q70" s="15"/>
+      <c r="R70" s="15"/>
+    </row>
+    <row r="71" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A71" s="15">
         <v>66</v>
       </c>
@@ -6132,8 +6270,10 @@
       <c r="P71" s="15">
         <v>17</v>
       </c>
-    </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q71" s="15"/>
+      <c r="R71" s="15"/>
+    </row>
+    <row r="72" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A72" s="15">
         <v>67</v>
       </c>
@@ -6174,8 +6314,10 @@
       <c r="P72" s="15">
         <v>17</v>
       </c>
-    </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q72" s="15"/>
+      <c r="R72" s="15"/>
+    </row>
+    <row r="73" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A73" s="15">
         <v>68</v>
       </c>
@@ -6216,8 +6358,10 @@
       <c r="P73" s="15">
         <v>17</v>
       </c>
-    </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q73" s="15"/>
+      <c r="R73" s="15"/>
+    </row>
+    <row r="74" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A74" s="5">
         <v>69</v>
       </c>
@@ -6260,8 +6404,10 @@
       <c r="P74" s="5">
         <v>17</v>
       </c>
-    </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q74" s="5"/>
+      <c r="R74" s="5"/>
+    </row>
+    <row r="75" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A75" s="5">
         <v>70</v>
       </c>
@@ -6304,8 +6450,10 @@
       <c r="P75" s="5">
         <v>16</v>
       </c>
-    </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q75" s="5"/>
+      <c r="R75" s="5"/>
+    </row>
+    <row r="76" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A76" s="5">
         <v>71</v>
       </c>
@@ -6346,8 +6494,10 @@
       <c r="P76" s="5">
         <v>16</v>
       </c>
-    </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q76" s="5"/>
+      <c r="R76" s="5"/>
+    </row>
+    <row r="77" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A77" s="5">
         <v>72</v>
       </c>
@@ -6390,8 +6540,10 @@
       <c r="P77" s="5">
         <v>16</v>
       </c>
-    </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q77" s="5"/>
+      <c r="R77" s="5"/>
+    </row>
+    <row r="78" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A78" s="5">
         <v>73</v>
       </c>
@@ -6434,8 +6586,10 @@
       <c r="P78" s="5">
         <v>16</v>
       </c>
-    </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q78" s="5"/>
+      <c r="R78" s="5"/>
+    </row>
+    <row r="79" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A79" s="5">
         <v>74</v>
       </c>
@@ -6478,8 +6632,10 @@
       <c r="P79" s="5">
         <v>16</v>
       </c>
-    </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q79" s="5"/>
+      <c r="R79" s="5"/>
+    </row>
+    <row r="80" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A80" s="5">
         <v>75</v>
       </c>
@@ -6522,8 +6678,10 @@
       <c r="P80" s="5">
         <v>16</v>
       </c>
-    </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q80" s="5"/>
+      <c r="R80" s="5"/>
+    </row>
+    <row r="81" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A81" s="5">
         <v>76</v>
       </c>
@@ -6566,8 +6724,10 @@
       <c r="P81" s="5">
         <v>16</v>
       </c>
-    </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q81" s="5"/>
+      <c r="R81" s="5"/>
+    </row>
+    <row r="82" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A82" s="5">
         <v>77</v>
       </c>
@@ -6610,8 +6770,10 @@
       <c r="P82" s="5">
         <v>16</v>
       </c>
-    </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q82" s="5"/>
+      <c r="R82" s="5"/>
+    </row>
+    <row r="83" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A83" s="15">
         <v>78</v>
       </c>
@@ -6650,8 +6812,10 @@
       <c r="P83" s="15">
         <v>16</v>
       </c>
-    </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q83" s="15"/>
+      <c r="R83" s="15"/>
+    </row>
+    <row r="84" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A84" s="15">
         <v>79</v>
       </c>
@@ -6690,8 +6854,10 @@
       <c r="P84" s="15">
         <v>16</v>
       </c>
-    </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q84" s="15"/>
+      <c r="R84" s="15"/>
+    </row>
+    <row r="85" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A85" s="5">
         <v>80</v>
       </c>
@@ -6732,8 +6898,10 @@
       <c r="N85" s="5"/>
       <c r="O85" s="5"/>
       <c r="P85" s="5"/>
-    </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q85" s="5"/>
+      <c r="R85" s="5"/>
+    </row>
+    <row r="86" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A86" s="5">
         <v>81</v>
       </c>
@@ -6774,8 +6942,10 @@
       <c r="N86" s="5"/>
       <c r="O86" s="5"/>
       <c r="P86" s="5"/>
-    </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q86" s="5"/>
+      <c r="R86" s="5"/>
+    </row>
+    <row r="87" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A87" s="5">
         <v>82</v>
       </c>
@@ -6816,8 +6986,10 @@
       <c r="N87" s="5"/>
       <c r="O87" s="5"/>
       <c r="P87" s="5"/>
-    </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q87" s="5"/>
+      <c r="R87" s="5"/>
+    </row>
+    <row r="88" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A88" s="5">
         <v>83</v>
       </c>
@@ -6858,8 +7030,10 @@
       <c r="N88" s="5"/>
       <c r="O88" s="5"/>
       <c r="P88" s="5"/>
-    </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q88" s="5"/>
+      <c r="R88" s="5"/>
+    </row>
+    <row r="89" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A89" s="5">
         <v>84</v>
       </c>
@@ -6900,8 +7074,10 @@
       <c r="N89" s="5"/>
       <c r="O89" s="5"/>
       <c r="P89" s="5"/>
-    </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q89" s="5"/>
+      <c r="R89" s="5"/>
+    </row>
+    <row r="90" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A90" s="5">
         <v>85</v>
       </c>
@@ -6944,8 +7120,10 @@
       <c r="N90" s="5"/>
       <c r="O90" s="5"/>
       <c r="P90" s="5"/>
-    </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q90" s="5"/>
+      <c r="R90" s="5"/>
+    </row>
+    <row r="91" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A91" s="5">
         <v>86</v>
       </c>
@@ -6988,8 +7166,10 @@
       <c r="N91" s="5"/>
       <c r="O91" s="5"/>
       <c r="P91" s="5"/>
-    </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q91" s="5"/>
+      <c r="R91" s="5"/>
+    </row>
+    <row r="92" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A92" s="5">
         <v>87</v>
       </c>
@@ -7032,8 +7212,10 @@
       <c r="N92" s="5"/>
       <c r="O92" s="5"/>
       <c r="P92" s="5"/>
-    </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q92" s="5"/>
+      <c r="R92" s="5"/>
+    </row>
+    <row r="93" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A93" s="5">
         <v>88</v>
       </c>
@@ -7076,8 +7258,10 @@
       <c r="N93" s="5"/>
       <c r="O93" s="5"/>
       <c r="P93" s="5"/>
-    </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q93" s="5"/>
+      <c r="R93" s="5"/>
+    </row>
+    <row r="94" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A94" s="5">
         <v>89</v>
       </c>
@@ -7118,8 +7302,10 @@
       <c r="N94" s="5"/>
       <c r="O94" s="5"/>
       <c r="P94" s="5"/>
-    </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q94" s="5"/>
+      <c r="R94" s="5"/>
+    </row>
+    <row r="95" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A95" s="5">
         <v>90</v>
       </c>
@@ -7160,8 +7346,10 @@
       <c r="N95" s="5"/>
       <c r="O95" s="5"/>
       <c r="P95" s="5"/>
-    </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q95" s="5"/>
+      <c r="R95" s="5"/>
+    </row>
+    <row r="96" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A96" s="15">
         <v>91</v>
       </c>
@@ -7196,8 +7384,10 @@
       <c r="N96" s="15"/>
       <c r="O96" s="15"/>
       <c r="P96" s="15"/>
-    </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q96" s="15"/>
+      <c r="R96" s="15"/>
+    </row>
+    <row r="97" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A97" s="15">
         <v>92</v>
       </c>
@@ -7228,8 +7418,10 @@
       <c r="N97" s="15"/>
       <c r="O97" s="15"/>
       <c r="P97" s="15"/>
-    </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q97" s="15"/>
+      <c r="R97" s="15"/>
+    </row>
+    <row r="98" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A98" s="6">
         <v>93</v>
       </c>
@@ -7258,8 +7450,10 @@
       <c r="N98" s="6"/>
       <c r="O98" s="6"/>
       <c r="P98" s="6"/>
-    </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q98" s="6"/>
+      <c r="R98" s="6"/>
+    </row>
+    <row r="99" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A99" s="6">
         <v>94</v>
       </c>
@@ -7288,8 +7482,10 @@
       <c r="N99" s="6"/>
       <c r="O99" s="6"/>
       <c r="P99" s="6"/>
-    </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q99" s="6"/>
+      <c r="R99" s="6"/>
+    </row>
+    <row r="100" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A100" s="6">
         <v>95</v>
       </c>
@@ -7318,8 +7514,10 @@
       <c r="N100" s="6"/>
       <c r="O100" s="6"/>
       <c r="P100" s="6"/>
-    </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q100" s="6"/>
+      <c r="R100" s="6"/>
+    </row>
+    <row r="101" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A101" s="6">
         <v>96</v>
       </c>
@@ -7348,8 +7546,10 @@
       <c r="N101" s="6"/>
       <c r="O101" s="6"/>
       <c r="P101" s="6"/>
-    </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q101" s="6"/>
+      <c r="R101" s="6"/>
+    </row>
+    <row r="102" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A102" s="6">
         <v>97</v>
       </c>
@@ -7378,8 +7578,10 @@
       <c r="N102" s="6"/>
       <c r="O102" s="6"/>
       <c r="P102" s="6"/>
-    </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q102" s="6"/>
+      <c r="R102" s="6"/>
+    </row>
+    <row r="103" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A103" s="6">
         <v>98</v>
       </c>
@@ -7408,8 +7610,10 @@
       <c r="N103" s="6"/>
       <c r="O103" s="6"/>
       <c r="P103" s="6"/>
-    </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q103" s="6"/>
+      <c r="R103" s="6"/>
+    </row>
+    <row r="104" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A104" s="6">
         <v>99</v>
       </c>
@@ -7438,8 +7642,10 @@
       <c r="N104" s="6"/>
       <c r="O104" s="6"/>
       <c r="P104" s="6"/>
-    </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q104" s="6"/>
+      <c r="R104" s="6"/>
+    </row>
+    <row r="105" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A105" s="6">
         <v>100</v>
       </c>
@@ -7468,8 +7674,10 @@
       <c r="N105" s="6"/>
       <c r="O105" s="6"/>
       <c r="P105" s="6"/>
-    </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q105" s="6"/>
+      <c r="R105" s="6"/>
+    </row>
+    <row r="106" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A106" s="6">
         <v>101</v>
       </c>
@@ -7498,8 +7706,10 @@
       <c r="N106" s="6"/>
       <c r="O106" s="6"/>
       <c r="P106" s="6"/>
-    </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q106" s="6"/>
+      <c r="R106" s="6"/>
+    </row>
+    <row r="107" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A107" s="6">
         <v>102</v>
       </c>
@@ -7528,8 +7738,10 @@
       <c r="N107" s="6"/>
       <c r="O107" s="6"/>
       <c r="P107" s="6"/>
-    </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q107" s="6"/>
+      <c r="R107" s="6"/>
+    </row>
+    <row r="108" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A108" s="6">
         <v>103</v>
       </c>
@@ -7558,8 +7770,10 @@
       <c r="N108" s="6"/>
       <c r="O108" s="6"/>
       <c r="P108" s="6"/>
-    </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q108" s="6"/>
+      <c r="R108" s="6"/>
+    </row>
+    <row r="109" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A109" s="6">
         <v>104</v>
       </c>
@@ -7588,8 +7802,10 @@
       <c r="N109" s="6"/>
       <c r="O109" s="6"/>
       <c r="P109" s="6"/>
-    </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q109" s="6"/>
+      <c r="R109" s="6"/>
+    </row>
+    <row r="110" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A110" s="6">
         <v>105</v>
       </c>
@@ -7618,8 +7834,10 @@
       <c r="N110" s="6"/>
       <c r="O110" s="6"/>
       <c r="P110" s="6"/>
-    </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q110" s="6"/>
+      <c r="R110" s="6"/>
+    </row>
+    <row r="111" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A111" s="6">
         <v>106</v>
       </c>
@@ -7648,8 +7866,10 @@
       <c r="N111" s="6"/>
       <c r="O111" s="6"/>
       <c r="P111" s="6"/>
-    </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q111" s="6"/>
+      <c r="R111" s="6"/>
+    </row>
+    <row r="112" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A112" s="6">
         <v>107</v>
       </c>
@@ -7678,8 +7898,10 @@
       <c r="N112" s="6"/>
       <c r="O112" s="6"/>
       <c r="P112" s="6"/>
-    </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q112" s="6"/>
+      <c r="R112" s="6"/>
+    </row>
+    <row r="113" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A113" s="6">
         <v>108</v>
       </c>
@@ -7708,8 +7930,10 @@
       <c r="N113" s="6"/>
       <c r="O113" s="6"/>
       <c r="P113" s="6"/>
-    </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q113" s="6"/>
+      <c r="R113" s="6"/>
+    </row>
+    <row r="114" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A114" s="6">
         <v>109</v>
       </c>
@@ -7738,8 +7962,10 @@
       <c r="N114" s="6"/>
       <c r="O114" s="6"/>
       <c r="P114" s="6"/>
-    </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q114" s="6"/>
+      <c r="R114" s="6"/>
+    </row>
+    <row r="115" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A115" s="6">
         <v>110</v>
       </c>
@@ -7768,8 +7994,10 @@
       <c r="N115" s="6"/>
       <c r="O115" s="6"/>
       <c r="P115" s="6"/>
-    </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q115" s="6"/>
+      <c r="R115" s="6"/>
+    </row>
+    <row r="116" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A116" s="6">
         <v>111</v>
       </c>
@@ -7798,8 +8026,10 @@
       <c r="N116" s="6"/>
       <c r="O116" s="6"/>
       <c r="P116" s="6"/>
-    </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q116" s="6"/>
+      <c r="R116" s="6"/>
+    </row>
+    <row r="117" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A117" s="6">
         <v>112</v>
       </c>
@@ -7828,8 +8058,10 @@
       <c r="N117" s="6"/>
       <c r="O117" s="6"/>
       <c r="P117" s="6"/>
-    </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q117" s="6"/>
+      <c r="R117" s="6"/>
+    </row>
+    <row r="118" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A118" s="6">
         <v>113</v>
       </c>
@@ -7858,8 +8090,10 @@
       <c r="N118" s="6"/>
       <c r="O118" s="6"/>
       <c r="P118" s="6"/>
-    </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q118" s="6"/>
+      <c r="R118" s="6"/>
+    </row>
+    <row r="119" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A119" s="6">
         <v>114</v>
       </c>
@@ -7888,8 +8122,10 @@
       <c r="N119" s="6"/>
       <c r="O119" s="6"/>
       <c r="P119" s="6"/>
-    </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q119" s="6"/>
+      <c r="R119" s="6"/>
+    </row>
+    <row r="120" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A120" s="6">
         <v>115</v>
       </c>
@@ -7918,8 +8154,10 @@
       <c r="N120" s="6"/>
       <c r="O120" s="6"/>
       <c r="P120" s="6"/>
-    </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q120" s="6"/>
+      <c r="R120" s="6"/>
+    </row>
+    <row r="121" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A121" s="6">
         <v>116</v>
       </c>
@@ -7948,8 +8186,10 @@
       <c r="N121" s="6"/>
       <c r="O121" s="6"/>
       <c r="P121" s="6"/>
-    </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q121" s="6"/>
+      <c r="R121" s="6"/>
+    </row>
+    <row r="122" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A122" s="6">
         <v>117</v>
       </c>
@@ -7978,8 +8218,10 @@
       <c r="N122" s="6"/>
       <c r="O122" s="6"/>
       <c r="P122" s="6"/>
-    </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q122" s="6"/>
+      <c r="R122" s="6"/>
+    </row>
+    <row r="123" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A123" s="6">
         <v>118</v>
       </c>
@@ -8008,8 +8250,10 @@
       <c r="N123" s="6"/>
       <c r="O123" s="6"/>
       <c r="P123" s="6"/>
-    </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q123" s="6"/>
+      <c r="R123" s="6"/>
+    </row>
+    <row r="124" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A124" s="6">
         <v>119</v>
       </c>
@@ -8038,8 +8282,10 @@
       <c r="N124" s="6"/>
       <c r="O124" s="6"/>
       <c r="P124" s="6"/>
-    </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q124" s="6"/>
+      <c r="R124" s="6"/>
+    </row>
+    <row r="125" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A125" s="6">
         <v>120</v>
       </c>
@@ -8068,8 +8314,10 @@
       <c r="N125" s="6"/>
       <c r="O125" s="6"/>
       <c r="P125" s="6"/>
-    </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q125" s="6"/>
+      <c r="R125" s="6"/>
+    </row>
+    <row r="126" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A126" s="6">
         <v>121</v>
       </c>
@@ -8098,8 +8346,10 @@
       <c r="N126" s="6"/>
       <c r="O126" s="6"/>
       <c r="P126" s="6"/>
-    </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q126" s="6"/>
+      <c r="R126" s="6"/>
+    </row>
+    <row r="127" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A127" s="6">
         <v>122</v>
       </c>
@@ -8128,8 +8378,10 @@
       <c r="N127" s="6"/>
       <c r="O127" s="6"/>
       <c r="P127" s="6"/>
-    </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q127" s="6"/>
+      <c r="R127" s="6"/>
+    </row>
+    <row r="128" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A128" s="6">
         <v>123</v>
       </c>
@@ -8158,8 +8410,10 @@
       <c r="N128" s="6"/>
       <c r="O128" s="6"/>
       <c r="P128" s="6"/>
-    </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q128" s="6"/>
+      <c r="R128" s="6"/>
+    </row>
+    <row r="129" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A129" s="6">
         <v>124</v>
       </c>
@@ -8188,8 +8442,10 @@
       <c r="N129" s="6"/>
       <c r="O129" s="6"/>
       <c r="P129" s="6"/>
-    </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q129" s="6"/>
+      <c r="R129" s="6"/>
+    </row>
+    <row r="130" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A130" s="6">
         <v>125</v>
       </c>
@@ -8218,8 +8474,10 @@
       <c r="N130" s="6"/>
       <c r="O130" s="6"/>
       <c r="P130" s="6"/>
-    </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q130" s="6"/>
+      <c r="R130" s="6"/>
+    </row>
+    <row r="131" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A131" s="6">
         <v>126</v>
       </c>
@@ -8248,8 +8506,10 @@
       <c r="N131" s="6"/>
       <c r="O131" s="6"/>
       <c r="P131" s="6"/>
-    </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q131" s="6"/>
+      <c r="R131" s="6"/>
+    </row>
+    <row r="132" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A132" s="6">
         <v>127</v>
       </c>
@@ -8278,8 +8538,10 @@
       <c r="N132" s="6"/>
       <c r="O132" s="6"/>
       <c r="P132" s="6"/>
-    </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q132" s="6"/>
+      <c r="R132" s="6"/>
+    </row>
+    <row r="133" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A133" s="6">
         <v>128</v>
       </c>
@@ -8308,8 +8570,10 @@
       <c r="N133" s="6"/>
       <c r="O133" s="6"/>
       <c r="P133" s="6"/>
-    </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q133" s="6"/>
+      <c r="R133" s="6"/>
+    </row>
+    <row r="134" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A134" s="6">
         <v>129</v>
       </c>
@@ -8338,8 +8602,10 @@
       <c r="N134" s="6"/>
       <c r="O134" s="6"/>
       <c r="P134" s="6"/>
-    </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q134" s="6"/>
+      <c r="R134" s="6"/>
+    </row>
+    <row r="135" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A135" s="6">
         <v>130</v>
       </c>
@@ -8368,8 +8634,10 @@
       <c r="N135" s="6"/>
       <c r="O135" s="6"/>
       <c r="P135" s="6"/>
-    </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q135" s="6"/>
+      <c r="R135" s="6"/>
+    </row>
+    <row r="136" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A136" s="6">
         <v>131</v>
       </c>
@@ -8398,8 +8666,10 @@
       <c r="N136" s="6"/>
       <c r="O136" s="6"/>
       <c r="P136" s="6"/>
-    </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q136" s="6"/>
+      <c r="R136" s="6"/>
+    </row>
+    <row r="137" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A137" s="6">
         <v>132</v>
       </c>
@@ -8428,8 +8698,10 @@
       <c r="N137" s="6"/>
       <c r="O137" s="6"/>
       <c r="P137" s="6"/>
-    </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q137" s="6"/>
+      <c r="R137" s="6"/>
+    </row>
+    <row r="138" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A138" s="6">
         <v>133</v>
       </c>
@@ -8458,8 +8730,10 @@
       <c r="N138" s="6"/>
       <c r="O138" s="6"/>
       <c r="P138" s="6"/>
-    </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q138" s="6"/>
+      <c r="R138" s="6"/>
+    </row>
+    <row r="139" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A139" s="6">
         <v>134</v>
       </c>
@@ -8488,8 +8762,10 @@
       <c r="N139" s="6"/>
       <c r="O139" s="6"/>
       <c r="P139" s="6"/>
-    </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q139" s="6"/>
+      <c r="R139" s="6"/>
+    </row>
+    <row r="140" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A140" s="6">
         <v>135</v>
       </c>
@@ -8518,8 +8794,10 @@
       <c r="N140" s="6"/>
       <c r="O140" s="6"/>
       <c r="P140" s="6"/>
-    </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q140" s="6"/>
+      <c r="R140" s="6"/>
+    </row>
+    <row r="141" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A141" s="6">
         <v>136</v>
       </c>
@@ -8548,8 +8826,10 @@
       <c r="N141" s="6"/>
       <c r="O141" s="6"/>
       <c r="P141" s="6"/>
-    </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q141" s="6"/>
+      <c r="R141" s="6"/>
+    </row>
+    <row r="142" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A142" s="6">
         <v>137</v>
       </c>
@@ -8578,8 +8858,10 @@
       <c r="N142" s="6"/>
       <c r="O142" s="6"/>
       <c r="P142" s="6"/>
-    </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q142" s="6"/>
+      <c r="R142" s="6"/>
+    </row>
+    <row r="143" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A143" s="6">
         <v>138</v>
       </c>
@@ -8608,8 +8890,10 @@
       <c r="N143" s="6"/>
       <c r="O143" s="6"/>
       <c r="P143" s="6"/>
-    </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q143" s="6"/>
+      <c r="R143" s="6"/>
+    </row>
+    <row r="144" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A144" s="6">
         <v>139</v>
       </c>
@@ -8638,8 +8922,10 @@
       <c r="N144" s="6"/>
       <c r="O144" s="6"/>
       <c r="P144" s="6"/>
-    </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q144" s="6"/>
+      <c r="R144" s="6"/>
+    </row>
+    <row r="145" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A145" s="6">
         <v>140</v>
       </c>
@@ -8668,8 +8954,10 @@
       <c r="N145" s="6"/>
       <c r="O145" s="6"/>
       <c r="P145" s="6"/>
-    </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q145" s="6"/>
+      <c r="R145" s="6"/>
+    </row>
+    <row r="146" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A146" s="6">
         <v>141</v>
       </c>
@@ -8698,8 +8986,10 @@
       <c r="N146" s="6"/>
       <c r="O146" s="6"/>
       <c r="P146" s="6"/>
-    </row>
-    <row r="147" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q146" s="6"/>
+      <c r="R146" s="6"/>
+    </row>
+    <row r="147" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A147" s="6">
         <v>142</v>
       </c>
@@ -8728,8 +9018,10 @@
       <c r="N147" s="6"/>
       <c r="O147" s="6"/>
       <c r="P147" s="6"/>
-    </row>
-    <row r="148" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q147" s="6"/>
+      <c r="R147" s="6"/>
+    </row>
+    <row r="148" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A148" s="6">
         <v>143</v>
       </c>
@@ -8758,8 +9050,10 @@
       <c r="N148" s="6"/>
       <c r="O148" s="6"/>
       <c r="P148" s="6"/>
-    </row>
-    <row r="149" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q148" s="6"/>
+      <c r="R148" s="6"/>
+    </row>
+    <row r="149" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A149" s="6">
         <v>144</v>
       </c>
@@ -8788,8 +9082,10 @@
       <c r="N149" s="6"/>
       <c r="O149" s="6"/>
       <c r="P149" s="6"/>
-    </row>
-    <row r="150" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q149" s="6"/>
+      <c r="R149" s="6"/>
+    </row>
+    <row r="150" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A150" s="6">
         <v>145</v>
       </c>
@@ -8818,8 +9114,10 @@
       <c r="N150" s="6"/>
       <c r="O150" s="6"/>
       <c r="P150" s="6"/>
-    </row>
-    <row r="151" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q150" s="6"/>
+      <c r="R150" s="6"/>
+    </row>
+    <row r="151" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A151" s="6">
         <v>146</v>
       </c>
@@ -8848,8 +9146,10 @@
       <c r="N151" s="6"/>
       <c r="O151" s="6"/>
       <c r="P151" s="6"/>
-    </row>
-    <row r="152" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q151" s="6"/>
+      <c r="R151" s="6"/>
+    </row>
+    <row r="152" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A152" s="6">
         <v>147</v>
       </c>
@@ -8878,8 +9178,10 @@
       <c r="N152" s="6"/>
       <c r="O152" s="6"/>
       <c r="P152" s="6"/>
-    </row>
-    <row r="153" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q152" s="6"/>
+      <c r="R152" s="6"/>
+    </row>
+    <row r="153" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A153" s="6">
         <v>148</v>
       </c>
@@ -8908,8 +9210,10 @@
       <c r="N153" s="6"/>
       <c r="O153" s="6"/>
       <c r="P153" s="6"/>
-    </row>
-    <row r="154" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q153" s="6"/>
+      <c r="R153" s="6"/>
+    </row>
+    <row r="154" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A154" s="6">
         <v>149</v>
       </c>
@@ -8938,8 +9242,10 @@
       <c r="N154" s="6"/>
       <c r="O154" s="6"/>
       <c r="P154" s="6"/>
-    </row>
-    <row r="155" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q154" s="6"/>
+      <c r="R154" s="6"/>
+    </row>
+    <row r="155" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A155" s="6">
         <v>150</v>
       </c>
@@ -8968,8 +9274,10 @@
       <c r="N155" s="6"/>
       <c r="O155" s="6"/>
       <c r="P155" s="6"/>
-    </row>
-    <row r="156" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q155" s="6"/>
+      <c r="R155" s="6"/>
+    </row>
+    <row r="156" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A156" s="6">
         <v>151</v>
       </c>
@@ -8998,8 +9306,10 @@
       <c r="N156" s="6"/>
       <c r="O156" s="6"/>
       <c r="P156" s="6"/>
-    </row>
-    <row r="157" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q156" s="6"/>
+      <c r="R156" s="6"/>
+    </row>
+    <row r="157" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A157" s="6">
         <v>152</v>
       </c>
@@ -9028,8 +9338,10 @@
       <c r="N157" s="6"/>
       <c r="O157" s="6"/>
       <c r="P157" s="6"/>
-    </row>
-    <row r="158" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q157" s="6"/>
+      <c r="R157" s="6"/>
+    </row>
+    <row r="158" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A158" s="6">
         <v>153</v>
       </c>
@@ -9058,8 +9370,10 @@
       <c r="N158" s="6"/>
       <c r="O158" s="6"/>
       <c r="P158" s="6"/>
-    </row>
-    <row r="159" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q158" s="6"/>
+      <c r="R158" s="6"/>
+    </row>
+    <row r="159" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A159" s="6">
         <v>154</v>
       </c>
@@ -9088,8 +9402,10 @@
       <c r="N159" s="6"/>
       <c r="O159" s="6"/>
       <c r="P159" s="6"/>
-    </row>
-    <row r="160" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q159" s="6"/>
+      <c r="R159" s="6"/>
+    </row>
+    <row r="160" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A160" s="6">
         <v>155</v>
       </c>
@@ -9118,8 +9434,10 @@
       <c r="N160" s="6"/>
       <c r="O160" s="6"/>
       <c r="P160" s="6"/>
-    </row>
-    <row r="161" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q160" s="6"/>
+      <c r="R160" s="6"/>
+    </row>
+    <row r="161" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A161" s="6">
         <v>156</v>
       </c>
@@ -9148,8 +9466,10 @@
       <c r="N161" s="6"/>
       <c r="O161" s="6"/>
       <c r="P161" s="6"/>
-    </row>
-    <row r="162" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q161" s="6"/>
+      <c r="R161" s="6"/>
+    </row>
+    <row r="162" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A162" s="6">
         <v>157</v>
       </c>
@@ -9178,8 +9498,10 @@
       <c r="N162" s="6"/>
       <c r="O162" s="6"/>
       <c r="P162" s="6"/>
-    </row>
-    <row r="163" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q162" s="6"/>
+      <c r="R162" s="6"/>
+    </row>
+    <row r="163" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A163" s="6">
         <v>158</v>
       </c>
@@ -9208,8 +9530,10 @@
       <c r="N163" s="6"/>
       <c r="O163" s="6"/>
       <c r="P163" s="6"/>
-    </row>
-    <row r="164" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q163" s="6"/>
+      <c r="R163" s="6"/>
+    </row>
+    <row r="164" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A164" s="6">
         <v>159</v>
       </c>
@@ -9238,8 +9562,10 @@
       <c r="N164" s="6"/>
       <c r="O164" s="6"/>
       <c r="P164" s="6"/>
-    </row>
-    <row r="165" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q164" s="6"/>
+      <c r="R164" s="6"/>
+    </row>
+    <row r="165" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A165" s="6">
         <v>160</v>
       </c>
@@ -9268,8 +9594,10 @@
       <c r="N165" s="6"/>
       <c r="O165" s="6"/>
       <c r="P165" s="6"/>
-    </row>
-    <row r="166" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q165" s="6"/>
+      <c r="R165" s="6"/>
+    </row>
+    <row r="166" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A166" s="6">
         <v>161</v>
       </c>
@@ -9298,8 +9626,10 @@
       <c r="N166" s="6"/>
       <c r="O166" s="6"/>
       <c r="P166" s="6"/>
-    </row>
-    <row r="167" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q166" s="6"/>
+      <c r="R166" s="6"/>
+    </row>
+    <row r="167" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A167" s="6">
         <v>162</v>
       </c>
@@ -9328,8 +9658,10 @@
       <c r="N167" s="6"/>
       <c r="O167" s="6"/>
       <c r="P167" s="6"/>
-    </row>
-    <row r="168" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q167" s="6"/>
+      <c r="R167" s="6"/>
+    </row>
+    <row r="168" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A168" s="6">
         <v>163</v>
       </c>
@@ -9358,8 +9690,10 @@
       <c r="N168" s="6"/>
       <c r="O168" s="6"/>
       <c r="P168" s="6"/>
-    </row>
-    <row r="169" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q168" s="6"/>
+      <c r="R168" s="6"/>
+    </row>
+    <row r="169" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A169" s="6">
         <v>164</v>
       </c>
@@ -9388,8 +9722,10 @@
       <c r="N169" s="6"/>
       <c r="O169" s="6"/>
       <c r="P169" s="6"/>
-    </row>
-    <row r="170" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q169" s="6"/>
+      <c r="R169" s="6"/>
+    </row>
+    <row r="170" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A170" s="6">
         <v>165</v>
       </c>
@@ -9418,8 +9754,10 @@
       <c r="N170" s="6"/>
       <c r="O170" s="6"/>
       <c r="P170" s="6"/>
-    </row>
-    <row r="171" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q170" s="6"/>
+      <c r="R170" s="6"/>
+    </row>
+    <row r="171" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A171" s="6">
         <v>166</v>
       </c>
@@ -9448,8 +9786,10 @@
       <c r="N171" s="6"/>
       <c r="O171" s="6"/>
       <c r="P171" s="6"/>
-    </row>
-    <row r="172" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q171" s="6"/>
+      <c r="R171" s="6"/>
+    </row>
+    <row r="172" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A172" s="6">
         <v>167</v>
       </c>
@@ -9478,8 +9818,10 @@
       <c r="N172" s="6"/>
       <c r="O172" s="6"/>
       <c r="P172" s="6"/>
-    </row>
-    <row r="173" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q172" s="6"/>
+      <c r="R172" s="6"/>
+    </row>
+    <row r="173" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A173" s="6">
         <v>168</v>
       </c>
@@ -9508,8 +9850,10 @@
       <c r="N173" s="6"/>
       <c r="O173" s="6"/>
       <c r="P173" s="6"/>
-    </row>
-    <row r="174" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q173" s="6"/>
+      <c r="R173" s="6"/>
+    </row>
+    <row r="174" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A174" s="6">
         <v>169</v>
       </c>
@@ -9538,8 +9882,10 @@
       <c r="N174" s="6"/>
       <c r="O174" s="6"/>
       <c r="P174" s="6"/>
-    </row>
-    <row r="175" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q174" s="6"/>
+      <c r="R174" s="6"/>
+    </row>
+    <row r="175" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A175" s="6">
         <v>170</v>
       </c>
@@ -9568,8 +9914,10 @@
       <c r="N175" s="6"/>
       <c r="O175" s="6"/>
       <c r="P175" s="6"/>
-    </row>
-    <row r="176" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q175" s="6"/>
+      <c r="R175" s="6"/>
+    </row>
+    <row r="176" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A176" s="6">
         <v>171</v>
       </c>
@@ -9598,8 +9946,10 @@
       <c r="N176" s="6"/>
       <c r="O176" s="6"/>
       <c r="P176" s="6"/>
-    </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q176" s="6"/>
+      <c r="R176" s="6"/>
+    </row>
+    <row r="177" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A177" s="6">
         <v>172</v>
       </c>
@@ -9628,8 +9978,10 @@
       <c r="N177" s="6"/>
       <c r="O177" s="6"/>
       <c r="P177" s="6"/>
-    </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q177" s="6"/>
+      <c r="R177" s="6"/>
+    </row>
+    <row r="178" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A178" s="6">
         <v>173</v>
       </c>
@@ -9658,8 +10010,10 @@
       <c r="N178" s="6"/>
       <c r="O178" s="6"/>
       <c r="P178" s="6"/>
-    </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q178" s="6"/>
+      <c r="R178" s="6"/>
+    </row>
+    <row r="179" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A179" s="6">
         <v>174</v>
       </c>
@@ -9688,8 +10042,10 @@
       <c r="N179" s="6"/>
       <c r="O179" s="6"/>
       <c r="P179" s="6"/>
-    </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q179" s="6"/>
+      <c r="R179" s="6"/>
+    </row>
+    <row r="180" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A180" s="6">
         <v>175</v>
       </c>
@@ -9718,8 +10074,10 @@
       <c r="N180" s="6"/>
       <c r="O180" s="6"/>
       <c r="P180" s="6"/>
-    </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q180" s="6"/>
+      <c r="R180" s="6"/>
+    </row>
+    <row r="181" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A181" s="6">
         <v>176</v>
       </c>
@@ -9748,8 +10106,10 @@
       <c r="N181" s="6"/>
       <c r="O181" s="6"/>
       <c r="P181" s="6"/>
-    </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q181" s="6"/>
+      <c r="R181" s="6"/>
+    </row>
+    <row r="182" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A182" s="6">
         <v>177</v>
       </c>
@@ -9778,8 +10138,10 @@
       <c r="N182" s="6"/>
       <c r="O182" s="6"/>
       <c r="P182" s="6"/>
-    </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q182" s="6"/>
+      <c r="R182" s="6"/>
+    </row>
+    <row r="183" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A183" s="6">
         <v>178</v>
       </c>
@@ -9808,8 +10170,10 @@
       <c r="N183" s="6"/>
       <c r="O183" s="6"/>
       <c r="P183" s="6"/>
-    </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q183" s="6"/>
+      <c r="R183" s="6"/>
+    </row>
+    <row r="184" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A184" s="6">
         <v>179</v>
       </c>
@@ -9838,8 +10202,10 @@
       <c r="N184" s="6"/>
       <c r="O184" s="6"/>
       <c r="P184" s="6"/>
-    </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q184" s="6"/>
+      <c r="R184" s="6"/>
+    </row>
+    <row r="185" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A185" s="6">
         <v>180</v>
       </c>
@@ -9868,8 +10234,10 @@
       <c r="N185" s="6"/>
       <c r="O185" s="6"/>
       <c r="P185" s="6"/>
-    </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q185" s="6"/>
+      <c r="R185" s="6"/>
+    </row>
+    <row r="186" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A186" s="6">
         <v>181</v>
       </c>
@@ -9898,8 +10266,10 @@
       <c r="N186" s="6"/>
       <c r="O186" s="6"/>
       <c r="P186" s="6"/>
-    </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q186" s="6"/>
+      <c r="R186" s="6"/>
+    </row>
+    <row r="187" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A187" s="7">
         <v>182</v>
       </c>
@@ -9930,8 +10300,10 @@
         <v>715</v>
       </c>
       <c r="P187" s="7"/>
-    </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q187" s="7"/>
+      <c r="R187" s="7"/>
+    </row>
+    <row r="188" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A188" s="7">
         <v>183</v>
       </c>
@@ -9958,8 +10330,10 @@
       <c r="N188" s="7"/>
       <c r="O188" s="17"/>
       <c r="P188" s="7"/>
-    </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q188" s="7"/>
+      <c r="R188" s="7"/>
+    </row>
+    <row r="189" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A189" s="7">
         <v>184</v>
       </c>
@@ -9986,8 +10360,10 @@
       <c r="N189" s="7"/>
       <c r="O189" s="17"/>
       <c r="P189" s="7"/>
-    </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q189" s="7"/>
+      <c r="R189" s="7"/>
+    </row>
+    <row r="190" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A190" s="7">
         <v>185</v>
       </c>
@@ -10014,8 +10390,10 @@
       <c r="N190" s="7"/>
       <c r="O190" s="17"/>
       <c r="P190" s="7"/>
-    </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q190" s="7"/>
+      <c r="R190" s="7"/>
+    </row>
+    <row r="191" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A191" s="7">
         <v>186</v>
       </c>
@@ -10054,8 +10432,10 @@
         <v>715</v>
       </c>
       <c r="P191" s="7"/>
-    </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q191" s="7"/>
+      <c r="R191" s="7"/>
+    </row>
+    <row r="192" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A192" s="7">
         <v>187</v>
       </c>
@@ -10094,8 +10474,10 @@
         <v>715</v>
       </c>
       <c r="P192" s="7"/>
-    </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q192" s="7"/>
+      <c r="R192" s="7"/>
+    </row>
+    <row r="193" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A193" s="7">
         <v>188</v>
       </c>
@@ -10134,8 +10516,10 @@
         <v>715</v>
       </c>
       <c r="P193" s="7"/>
-    </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q193" s="7"/>
+      <c r="R193" s="7"/>
+    </row>
+    <row r="194" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A194" s="7">
         <v>189</v>
       </c>
@@ -10164,8 +10548,10 @@
         <v>715</v>
       </c>
       <c r="P194" s="7"/>
-    </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q194" s="7"/>
+      <c r="R194" s="7"/>
+    </row>
+    <row r="195" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A195" s="7">
         <v>190</v>
       </c>
@@ -10200,8 +10586,10 @@
       <c r="N195" s="7"/>
       <c r="O195" s="13"/>
       <c r="P195" s="7"/>
-    </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q195" s="7"/>
+      <c r="R195" s="7"/>
+    </row>
+    <row r="196" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A196" s="7">
         <v>191</v>
       </c>
@@ -10232,8 +10620,10 @@
         <v>715</v>
       </c>
       <c r="P196" s="7"/>
-    </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q196" s="7"/>
+      <c r="R196" s="7"/>
+    </row>
+    <row r="197" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A197" s="7">
         <v>192</v>
       </c>
@@ -10264,8 +10654,10 @@
         <v>715</v>
       </c>
       <c r="P197" s="7"/>
-    </row>
-    <row r="198" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q197" s="7"/>
+      <c r="R197" s="7"/>
+    </row>
+    <row r="198" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A198" s="7">
         <v>193</v>
       </c>
@@ -10296,8 +10688,10 @@
         <v>715</v>
       </c>
       <c r="P198" s="7"/>
-    </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q198" s="7"/>
+      <c r="R198" s="7"/>
+    </row>
+    <row r="199" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A199" s="7">
         <v>194</v>
       </c>
@@ -10328,8 +10722,10 @@
         <v>715</v>
       </c>
       <c r="P199" s="7"/>
-    </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q199" s="7"/>
+      <c r="R199" s="7"/>
+    </row>
+    <row r="200" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A200" s="7">
         <v>195</v>
       </c>
@@ -10360,8 +10756,10 @@
         <v>715</v>
       </c>
       <c r="P200" s="7"/>
-    </row>
-    <row r="201" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q200" s="7"/>
+      <c r="R200" s="7"/>
+    </row>
+    <row r="201" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A201" s="7">
         <v>196</v>
       </c>
@@ -10392,8 +10790,10 @@
         <v>715</v>
       </c>
       <c r="P201" s="7"/>
-    </row>
-    <row r="202" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q201" s="7"/>
+      <c r="R201" s="7"/>
+    </row>
+    <row r="202" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A202" s="7">
         <v>197</v>
       </c>
@@ -10424,8 +10824,10 @@
         <v>715</v>
       </c>
       <c r="P202" s="7"/>
-    </row>
-    <row r="203" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q202" s="7"/>
+      <c r="R202" s="7"/>
+    </row>
+    <row r="203" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A203" s="7">
         <v>198</v>
       </c>
@@ -10456,8 +10858,10 @@
         <v>715</v>
       </c>
       <c r="P203" s="7"/>
-    </row>
-    <row r="204" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q203" s="7"/>
+      <c r="R203" s="7"/>
+    </row>
+    <row r="204" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A204" s="7">
         <v>199</v>
       </c>
@@ -10488,8 +10892,10 @@
         <v>715</v>
       </c>
       <c r="P204" s="7"/>
-    </row>
-    <row r="205" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q204" s="7"/>
+      <c r="R204" s="7"/>
+    </row>
+    <row r="205" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A205" s="7">
         <v>200</v>
       </c>
@@ -10520,8 +10926,10 @@
         <v>715</v>
       </c>
       <c r="P205" s="7"/>
-    </row>
-    <row r="206" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q205" s="7"/>
+      <c r="R205" s="7"/>
+    </row>
+    <row r="206" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A206" s="7">
         <v>201</v>
       </c>
@@ -10548,8 +10956,10 @@
       <c r="N206" s="7"/>
       <c r="O206" s="13"/>
       <c r="P206" s="7"/>
-    </row>
-    <row r="207" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q206" s="7"/>
+      <c r="R206" s="7"/>
+    </row>
+    <row r="207" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A207" s="7">
         <v>202</v>
       </c>
@@ -10576,8 +10986,10 @@
       <c r="N207" s="7"/>
       <c r="O207" s="13"/>
       <c r="P207" s="7"/>
-    </row>
-    <row r="208" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q207" s="7"/>
+      <c r="R207" s="7"/>
+    </row>
+    <row r="208" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A208" s="7">
         <v>203</v>
       </c>
@@ -10604,8 +11016,10 @@
       <c r="N208" s="7"/>
       <c r="O208" s="13"/>
       <c r="P208" s="7"/>
-    </row>
-    <row r="209" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q208" s="7"/>
+      <c r="R208" s="7"/>
+    </row>
+    <row r="209" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A209" s="7">
         <v>204</v>
       </c>
@@ -10632,8 +11046,10 @@
       <c r="N209" s="7"/>
       <c r="O209" s="13"/>
       <c r="P209" s="7"/>
-    </row>
-    <row r="210" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q209" s="7"/>
+      <c r="R209" s="7"/>
+    </row>
+    <row r="210" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A210" s="7">
         <v>205</v>
       </c>
@@ -10660,8 +11076,10 @@
       <c r="N210" s="7"/>
       <c r="O210" s="13"/>
       <c r="P210" s="7"/>
-    </row>
-    <row r="211" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q210" s="7"/>
+      <c r="R210" s="7"/>
+    </row>
+    <row r="211" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A211" s="7">
         <v>206</v>
       </c>
@@ -10688,8 +11106,10 @@
       <c r="N211" s="7"/>
       <c r="O211" s="13"/>
       <c r="P211" s="7"/>
-    </row>
-    <row r="212" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q211" s="7"/>
+      <c r="R211" s="7"/>
+    </row>
+    <row r="212" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A212" s="7">
         <v>207</v>
       </c>
@@ -10716,8 +11136,10 @@
       <c r="N212" s="7"/>
       <c r="O212" s="13"/>
       <c r="P212" s="7"/>
-    </row>
-    <row r="213" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q212" s="7"/>
+      <c r="R212" s="7"/>
+    </row>
+    <row r="213" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A213" s="7">
         <v>208</v>
       </c>
@@ -10754,8 +11176,10 @@
       <c r="N213" s="7"/>
       <c r="O213" s="13"/>
       <c r="P213" s="7"/>
-    </row>
-    <row r="214" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q213" s="7"/>
+      <c r="R213" s="7"/>
+    </row>
+    <row r="214" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A214" s="7">
         <v>209</v>
       </c>
@@ -10784,8 +11208,10 @@
       <c r="N214" s="7"/>
       <c r="O214" s="13"/>
       <c r="P214" s="7"/>
-    </row>
-    <row r="215" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q214" s="7"/>
+      <c r="R214" s="7"/>
+    </row>
+    <row r="215" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A215" s="7">
         <v>210</v>
       </c>
@@ -10814,8 +11240,10 @@
       <c r="N215" s="7"/>
       <c r="O215" s="13"/>
       <c r="P215" s="7"/>
-    </row>
-    <row r="216" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q215" s="7"/>
+      <c r="R215" s="7"/>
+    </row>
+    <row r="216" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A216" s="7">
         <v>211</v>
       </c>
@@ -10844,8 +11272,10 @@
       <c r="N216" s="7"/>
       <c r="O216" s="13"/>
       <c r="P216" s="7"/>
-    </row>
-    <row r="217" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q216" s="7"/>
+      <c r="R216" s="7"/>
+    </row>
+    <row r="217" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A217" s="7">
         <v>212</v>
       </c>
@@ -10872,8 +11302,10 @@
       <c r="N217" s="7"/>
       <c r="O217" s="13"/>
       <c r="P217" s="7"/>
-    </row>
-    <row r="218" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q217" s="7"/>
+      <c r="R217" s="7"/>
+    </row>
+    <row r="218" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A218" s="7">
         <v>213</v>
       </c>
@@ -10902,8 +11334,10 @@
         <v>715</v>
       </c>
       <c r="P218" s="7"/>
-    </row>
-    <row r="219" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q218" s="7"/>
+      <c r="R218" s="7"/>
+    </row>
+    <row r="219" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A219" s="7">
         <v>214</v>
       </c>
@@ -10940,8 +11374,10 @@
         <v>715</v>
       </c>
       <c r="P219" s="7"/>
-    </row>
-    <row r="220" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q219" s="7"/>
+      <c r="R219" s="7"/>
+    </row>
+    <row r="220" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A220" s="7">
         <v>215</v>
       </c>
@@ -10972,8 +11408,10 @@
         <v>715</v>
       </c>
       <c r="P220" s="7"/>
-    </row>
-    <row r="221" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q220" s="7"/>
+      <c r="R220" s="7"/>
+    </row>
+    <row r="221" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A221" s="7">
         <v>216</v>
       </c>
@@ -11004,8 +11442,10 @@
         <v>715</v>
       </c>
       <c r="P221" s="7"/>
-    </row>
-    <row r="222" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q221" s="7"/>
+      <c r="R221" s="7"/>
+    </row>
+    <row r="222" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A222" s="7">
         <v>217</v>
       </c>
@@ -11044,8 +11484,10 @@
         <v>715</v>
       </c>
       <c r="P222" s="7"/>
-    </row>
-    <row r="223" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="Q222" s="7"/>
+      <c r="R222" s="7"/>
+    </row>
+    <row r="223" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A223" s="7">
         <v>218</v>
       </c>
@@ -11084,8 +11526,10 @@
         <v>715</v>
       </c>
       <c r="P223" s="7"/>
-    </row>
-    <row r="224" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q223" s="7"/>
+      <c r="R223" s="7"/>
+    </row>
+    <row r="224" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A224" s="7">
         <v>219</v>
       </c>
@@ -11124,8 +11568,10 @@
         <v>715</v>
       </c>
       <c r="P224" s="7"/>
-    </row>
-    <row r="225" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q224" s="7"/>
+      <c r="R224" s="7"/>
+    </row>
+    <row r="225" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A225" s="7">
         <v>220</v>
       </c>
@@ -11164,8 +11610,10 @@
         <v>715</v>
       </c>
       <c r="P225" s="7"/>
-    </row>
-    <row r="226" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q225" s="7"/>
+      <c r="R225" s="7"/>
+    </row>
+    <row r="226" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A226" s="7">
         <v>221</v>
       </c>
@@ -11204,8 +11652,10 @@
         <v>715</v>
       </c>
       <c r="P226" s="7"/>
-    </row>
-    <row r="227" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q226" s="7"/>
+      <c r="R226" s="7"/>
+    </row>
+    <row r="227" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A227" s="7">
         <v>222</v>
       </c>
@@ -11244,8 +11694,10 @@
         <v>715</v>
       </c>
       <c r="P227" s="7"/>
-    </row>
-    <row r="228" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q227" s="7"/>
+      <c r="R227" s="7"/>
+    </row>
+    <row r="228" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A228" s="7">
         <v>223</v>
       </c>
@@ -11284,8 +11736,10 @@
         <v>715</v>
       </c>
       <c r="P228" s="7"/>
-    </row>
-    <row r="229" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q228" s="7"/>
+      <c r="R228" s="7"/>
+    </row>
+    <row r="229" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A229" s="7">
         <v>224</v>
       </c>
@@ -11324,8 +11778,10 @@
         <v>715</v>
       </c>
       <c r="P229" s="7"/>
-    </row>
-    <row r="230" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q229" s="7"/>
+      <c r="R229" s="7"/>
+    </row>
+    <row r="230" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A230" s="7">
         <v>225</v>
       </c>
@@ -11364,8 +11820,10 @@
         <v>715</v>
       </c>
       <c r="P230" s="7"/>
-    </row>
-    <row r="231" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q230" s="7"/>
+      <c r="R230" s="7"/>
+    </row>
+    <row r="231" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A231" s="7">
         <v>226</v>
       </c>
@@ -11404,8 +11862,10 @@
         <v>715</v>
       </c>
       <c r="P231" s="7"/>
-    </row>
-    <row r="232" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q231" s="7"/>
+      <c r="R231" s="7"/>
+    </row>
+    <row r="232" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A232" s="7">
         <v>227</v>
       </c>
@@ -11444,8 +11904,10 @@
         <v>715</v>
       </c>
       <c r="P232" s="7"/>
-    </row>
-    <row r="233" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q232" s="7"/>
+      <c r="R232" s="7"/>
+    </row>
+    <row r="233" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A233" s="7">
         <v>228</v>
       </c>
@@ -11474,8 +11936,10 @@
       <c r="N233" s="7"/>
       <c r="O233" s="13"/>
       <c r="P233" s="7"/>
-    </row>
-    <row r="234" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q233" s="7"/>
+      <c r="R233" s="7"/>
+    </row>
+    <row r="234" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A234" s="7">
         <v>229</v>
       </c>
@@ -11510,8 +11974,10 @@
       <c r="N234" s="7"/>
       <c r="O234" s="13"/>
       <c r="P234" s="7"/>
-    </row>
-    <row r="235" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q234" s="7"/>
+      <c r="R234" s="7"/>
+    </row>
+    <row r="235" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A235" s="7">
         <v>230</v>
       </c>
@@ -11540,8 +12006,10 @@
         <v>715</v>
       </c>
       <c r="P235" s="7"/>
-    </row>
-    <row r="236" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q235" s="7"/>
+      <c r="R235" s="7"/>
+    </row>
+    <row r="236" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A236" s="7">
         <v>231</v>
       </c>
@@ -11572,8 +12040,10 @@
         <v>715</v>
       </c>
       <c r="P236" s="7"/>
-    </row>
-    <row r="237" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q236" s="7"/>
+      <c r="R236" s="7"/>
+    </row>
+    <row r="237" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A237" s="7">
         <v>232</v>
       </c>
@@ -11602,8 +12072,10 @@
       <c r="N237" s="7"/>
       <c r="O237" s="13"/>
       <c r="P237" s="7"/>
-    </row>
-    <row r="238" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q237" s="7"/>
+      <c r="R237" s="7"/>
+    </row>
+    <row r="238" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A238" s="7">
         <v>233</v>
       </c>
@@ -11632,8 +12104,10 @@
       <c r="N238" s="7"/>
       <c r="O238" s="13"/>
       <c r="P238" s="7"/>
-    </row>
-    <row r="239" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q238" s="7"/>
+      <c r="R238" s="7"/>
+    </row>
+    <row r="239" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A239" s="7">
         <v>234</v>
       </c>
@@ -11664,8 +12138,10 @@
         <v>715</v>
       </c>
       <c r="P239" s="7"/>
-    </row>
-    <row r="240" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q239" s="7"/>
+      <c r="R239" s="7"/>
+    </row>
+    <row r="240" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A240" s="7">
         <v>235</v>
       </c>
@@ -11694,8 +12170,10 @@
         <v>715</v>
       </c>
       <c r="P240" s="7"/>
-    </row>
-    <row r="241" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q240" s="7"/>
+      <c r="R240" s="7"/>
+    </row>
+    <row r="241" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A241" s="7">
         <v>236</v>
       </c>
@@ -11726,8 +12204,10 @@
         <v>716</v>
       </c>
       <c r="P241" s="7"/>
-    </row>
-    <row r="242" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q241" s="7"/>
+      <c r="R241" s="7"/>
+    </row>
+    <row r="242" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A242" s="7">
         <v>237</v>
       </c>
@@ -11758,8 +12238,10 @@
         <v>715</v>
       </c>
       <c r="P242" s="7"/>
-    </row>
-    <row r="243" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q242" s="7"/>
+      <c r="R242" s="7"/>
+    </row>
+    <row r="243" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A243" s="7">
         <v>238</v>
       </c>
@@ -11790,8 +12272,10 @@
         <v>716</v>
       </c>
       <c r="P243" s="7"/>
-    </row>
-    <row r="244" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q243" s="7"/>
+      <c r="R243" s="7"/>
+    </row>
+    <row r="244" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A244" s="7">
         <v>239</v>
       </c>
@@ -11822,8 +12306,10 @@
         <v>715</v>
       </c>
       <c r="P244" s="7"/>
-    </row>
-    <row r="245" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q244" s="7"/>
+      <c r="R244" s="7"/>
+    </row>
+    <row r="245" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A245" s="7">
         <v>240</v>
       </c>
@@ -11860,8 +12346,10 @@
         <v>716</v>
       </c>
       <c r="P245" s="7"/>
-    </row>
-    <row r="246" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q245" s="7"/>
+      <c r="R245" s="7"/>
+    </row>
+    <row r="246" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A246" s="7">
         <v>241</v>
       </c>
@@ -11892,8 +12380,10 @@
         <v>716</v>
       </c>
       <c r="P246" s="7"/>
-    </row>
-    <row r="247" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q246" s="7"/>
+      <c r="R246" s="7"/>
+    </row>
+    <row r="247" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A247" s="7">
         <v>242</v>
       </c>
@@ -11924,8 +12414,10 @@
         <v>715</v>
       </c>
       <c r="P247" s="7"/>
-    </row>
-    <row r="248" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q247" s="7"/>
+      <c r="R247" s="7"/>
+    </row>
+    <row r="248" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A248" s="7">
         <v>243</v>
       </c>
@@ -11956,8 +12448,10 @@
         <v>715</v>
       </c>
       <c r="P248" s="7"/>
-    </row>
-    <row r="249" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q248" s="7"/>
+      <c r="R248" s="7"/>
+    </row>
+    <row r="249" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A249" s="7">
         <v>244</v>
       </c>
@@ -11988,8 +12482,10 @@
         <v>716</v>
       </c>
       <c r="P249" s="7"/>
-    </row>
-    <row r="250" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q249" s="7"/>
+      <c r="R249" s="7"/>
+    </row>
+    <row r="250" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A250" s="7">
         <v>245</v>
       </c>
@@ -12018,8 +12514,10 @@
         <v>716</v>
       </c>
       <c r="P250" s="7"/>
-    </row>
-    <row r="251" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q250" s="7"/>
+      <c r="R250" s="7"/>
+    </row>
+    <row r="251" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A251" s="7">
         <v>246</v>
       </c>
@@ -12050,8 +12548,10 @@
         <v>716</v>
       </c>
       <c r="P251" s="7"/>
-    </row>
-    <row r="252" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q251" s="7"/>
+      <c r="R251" s="7"/>
+    </row>
+    <row r="252" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A252" s="7">
         <v>247</v>
       </c>
@@ -12080,8 +12580,10 @@
       <c r="N252" s="7"/>
       <c r="O252" s="13"/>
       <c r="P252" s="14"/>
-    </row>
-    <row r="253" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q252" s="7"/>
+      <c r="R252" s="7"/>
+    </row>
+    <row r="253" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A253" s="7">
         <v>248</v>
       </c>
@@ -12110,8 +12612,10 @@
       <c r="N253" s="7"/>
       <c r="O253" s="17"/>
       <c r="P253" s="14"/>
-    </row>
-    <row r="254" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q253" s="7"/>
+      <c r="R253" s="7"/>
+    </row>
+    <row r="254" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A254" s="7">
         <v>249</v>
       </c>
@@ -12142,8 +12646,10 @@
         <v>715</v>
       </c>
       <c r="P254" s="7"/>
-    </row>
-    <row r="255" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q254" s="7"/>
+      <c r="R254" s="7"/>
+    </row>
+    <row r="255" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A255" s="7">
         <v>250</v>
       </c>
@@ -12174,8 +12680,10 @@
         <v>715</v>
       </c>
       <c r="P255" s="7"/>
-    </row>
-    <row r="256" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q255" s="7"/>
+      <c r="R255" s="7"/>
+    </row>
+    <row r="256" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A256" s="7">
         <v>251</v>
       </c>
@@ -12206,8 +12714,10 @@
         <v>715</v>
       </c>
       <c r="P256" s="7"/>
-    </row>
-    <row r="257" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q256" s="7"/>
+      <c r="R256" s="7"/>
+    </row>
+    <row r="257" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A257" s="7">
         <v>252</v>
       </c>
@@ -12244,8 +12754,10 @@
         <v>715</v>
       </c>
       <c r="P257" s="7"/>
-    </row>
-    <row r="258" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q257" s="7"/>
+      <c r="R257" s="7"/>
+    </row>
+    <row r="258" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A258" s="7">
         <v>253</v>
       </c>
@@ -12276,8 +12788,10 @@
         <v>716</v>
       </c>
       <c r="P258" s="7"/>
-    </row>
-    <row r="259" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q258" s="7"/>
+      <c r="R258" s="7"/>
+    </row>
+    <row r="259" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A259" s="7">
         <v>254</v>
       </c>
@@ -12308,8 +12822,10 @@
         <v>716</v>
       </c>
       <c r="P259" s="7"/>
-    </row>
-    <row r="260" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q259" s="7"/>
+      <c r="R259" s="7"/>
+    </row>
+    <row r="260" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A260" s="7">
         <v>255</v>
       </c>
@@ -12338,8 +12854,10 @@
         <v>716</v>
       </c>
       <c r="P260" s="7"/>
-    </row>
-    <row r="261" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q260" s="7"/>
+      <c r="R260" s="7"/>
+    </row>
+    <row r="261" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A261" s="7">
         <v>256</v>
       </c>
@@ -12370,8 +12888,10 @@
         <v>716</v>
       </c>
       <c r="P261" s="7"/>
-    </row>
-    <row r="262" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q261" s="7"/>
+      <c r="R261" s="7"/>
+    </row>
+    <row r="262" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A262" s="7">
         <v>257</v>
       </c>
@@ -12402,8 +12922,10 @@
         <v>715</v>
       </c>
       <c r="P262" s="7"/>
-    </row>
-    <row r="263" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q262" s="7"/>
+      <c r="R262" s="7"/>
+    </row>
+    <row r="263" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A263" s="7">
         <v>258</v>
       </c>
@@ -12434,8 +12956,10 @@
         <v>716</v>
       </c>
       <c r="P263" s="7"/>
-    </row>
-    <row r="264" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q263" s="7"/>
+      <c r="R263" s="7"/>
+    </row>
+    <row r="264" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A264" s="7">
         <v>259</v>
       </c>
@@ -12472,8 +12996,10 @@
         <v>716</v>
       </c>
       <c r="P264" s="14"/>
-    </row>
-    <row r="265" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q264" s="7"/>
+      <c r="R264" s="7"/>
+    </row>
+    <row r="265" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A265" s="7">
         <v>260</v>
       </c>
@@ -12510,8 +13036,10 @@
         <v>716</v>
       </c>
       <c r="P265" s="14"/>
-    </row>
-    <row r="266" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q265" s="7"/>
+      <c r="R265" s="7"/>
+    </row>
+    <row r="266" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A266" s="7">
         <v>261</v>
       </c>
@@ -12548,8 +13076,10 @@
         <v>716</v>
       </c>
       <c r="P266" s="14"/>
-    </row>
-    <row r="267" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q266" s="7"/>
+      <c r="R266" s="7"/>
+    </row>
+    <row r="267" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A267" s="7">
         <v>262</v>
       </c>
@@ -12584,8 +13114,10 @@
         <v>716</v>
       </c>
       <c r="P267" s="14"/>
-    </row>
-    <row r="268" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q267" s="7"/>
+      <c r="R267" s="7"/>
+    </row>
+    <row r="268" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A268" s="7">
         <v>263</v>
       </c>
@@ -12614,8 +13146,10 @@
       <c r="N268" s="7"/>
       <c r="O268" s="13"/>
       <c r="P268" s="14"/>
-    </row>
-    <row r="269" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q268" s="7"/>
+      <c r="R268" s="7"/>
+    </row>
+    <row r="269" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A269" s="7">
         <v>264</v>
       </c>
@@ -12644,8 +13178,10 @@
       <c r="N269" s="7"/>
       <c r="O269" s="13"/>
       <c r="P269" s="14"/>
-    </row>
-    <row r="270" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q269" s="7"/>
+      <c r="R269" s="7"/>
+    </row>
+    <row r="270" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A270" s="7">
         <v>265</v>
       </c>
@@ -12674,8 +13210,10 @@
       <c r="N270" s="7"/>
       <c r="O270" s="13"/>
       <c r="P270" s="7"/>
-    </row>
-    <row r="271" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q270" s="7"/>
+      <c r="R270" s="7"/>
+    </row>
+    <row r="271" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A271" s="7">
         <v>266</v>
       </c>
@@ -12706,8 +13244,10 @@
         <v>715</v>
       </c>
       <c r="P271" s="7"/>
-    </row>
-    <row r="272" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q271" s="7"/>
+      <c r="R271" s="7"/>
+    </row>
+    <row r="272" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A272" s="7">
         <v>267</v>
       </c>
@@ -12736,8 +13276,10 @@
         <v>716</v>
       </c>
       <c r="P272" s="7"/>
-    </row>
-    <row r="273" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q272" s="7"/>
+      <c r="R272" s="7"/>
+    </row>
+    <row r="273" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A273" s="7">
         <v>268</v>
       </c>
@@ -12766,8 +13308,10 @@
         <v>716</v>
       </c>
       <c r="P273" s="7"/>
-    </row>
-    <row r="274" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q273" s="7"/>
+      <c r="R273" s="7"/>
+    </row>
+    <row r="274" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A274" s="7">
         <v>269</v>
       </c>
@@ -12798,8 +13342,10 @@
         <v>715</v>
       </c>
       <c r="P274" s="7"/>
-    </row>
-    <row r="275" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q274" s="7"/>
+      <c r="R274" s="7"/>
+    </row>
+    <row r="275" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A275" s="7">
         <v>270</v>
       </c>
@@ -12830,8 +13376,10 @@
         <v>715</v>
       </c>
       <c r="P275" s="7"/>
-    </row>
-    <row r="276" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q275" s="7"/>
+      <c r="R275" s="7"/>
+    </row>
+    <row r="276" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A276" s="7">
         <v>271</v>
       </c>
@@ -12862,8 +13410,10 @@
         <v>715</v>
       </c>
       <c r="P276" s="7"/>
-    </row>
-    <row r="277" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q276" s="7"/>
+      <c r="R276" s="7"/>
+    </row>
+    <row r="277" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A277" s="7">
         <v>272</v>
       </c>
@@ -12894,8 +13444,10 @@
         <v>715</v>
       </c>
       <c r="P277" s="7"/>
-    </row>
-    <row r="278" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q277" s="7"/>
+      <c r="R277" s="7"/>
+    </row>
+    <row r="278" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A278" s="7">
         <v>273</v>
       </c>
@@ -12926,8 +13478,10 @@
         <v>715</v>
       </c>
       <c r="P278" s="7"/>
-    </row>
-    <row r="279" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q278" s="7"/>
+      <c r="R278" s="7"/>
+    </row>
+    <row r="279" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A279" s="7">
         <v>274</v>
       </c>
@@ -12958,8 +13512,10 @@
         <v>715</v>
       </c>
       <c r="P279" s="7"/>
-    </row>
-    <row r="280" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q279" s="7"/>
+      <c r="R279" s="7"/>
+    </row>
+    <row r="280" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A280" s="7">
         <v>275</v>
       </c>
@@ -12994,8 +13550,10 @@
         <v>715</v>
       </c>
       <c r="P280" s="7"/>
-    </row>
-    <row r="281" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q280" s="7"/>
+      <c r="R280" s="7"/>
+    </row>
+    <row r="281" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A281" s="8">
         <v>276</v>
       </c>
@@ -13034,8 +13592,10 @@
       <c r="N281" s="8"/>
       <c r="O281" s="8"/>
       <c r="P281" s="8"/>
-    </row>
-    <row r="282" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q281" s="8"/>
+      <c r="R281" s="8"/>
+    </row>
+    <row r="282" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A282" s="8">
         <v>277</v>
       </c>
@@ -13076,8 +13636,10 @@
       <c r="N282" s="8"/>
       <c r="O282" s="8"/>
       <c r="P282" s="8"/>
-    </row>
-    <row r="283" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q282" s="8"/>
+      <c r="R282" s="8"/>
+    </row>
+    <row r="283" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A283" s="8">
         <v>278</v>
       </c>
@@ -13118,8 +13680,10 @@
       <c r="N283" s="8"/>
       <c r="O283" s="8"/>
       <c r="P283" s="8"/>
-    </row>
-    <row r="284" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q283" s="8"/>
+      <c r="R283" s="8"/>
+    </row>
+    <row r="284" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A284" s="8">
         <v>279</v>
       </c>
@@ -13160,8 +13724,10 @@
       <c r="N284" s="8"/>
       <c r="O284" s="8"/>
       <c r="P284" s="8"/>
-    </row>
-    <row r="285" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q284" s="8"/>
+      <c r="R284" s="8"/>
+    </row>
+    <row r="285" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A285" s="8">
         <v>280</v>
       </c>
@@ -13202,8 +13768,10 @@
       <c r="N285" s="8"/>
       <c r="O285" s="8"/>
       <c r="P285" s="8"/>
-    </row>
-    <row r="286" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q285" s="8"/>
+      <c r="R285" s="8"/>
+    </row>
+    <row r="286" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A286" s="8">
         <v>281</v>
       </c>
@@ -13244,8 +13812,10 @@
       <c r="N286" s="8"/>
       <c r="O286" s="8"/>
       <c r="P286" s="8"/>
-    </row>
-    <row r="287" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q286" s="8"/>
+      <c r="R286" s="8"/>
+    </row>
+    <row r="287" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A287" s="8">
         <v>282</v>
       </c>
@@ -13286,8 +13856,10 @@
       <c r="N287" s="8"/>
       <c r="O287" s="8"/>
       <c r="P287" s="8"/>
-    </row>
-    <row r="288" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q287" s="8"/>
+      <c r="R287" s="8"/>
+    </row>
+    <row r="288" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A288" s="8">
         <v>283</v>
       </c>
@@ -13330,8 +13902,10 @@
       <c r="N288" s="8"/>
       <c r="O288" s="8"/>
       <c r="P288" s="8"/>
-    </row>
-    <row r="289" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q288" s="8"/>
+      <c r="R288" s="8"/>
+    </row>
+    <row r="289" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A289" s="8">
         <v>284</v>
       </c>
@@ -13372,8 +13946,10 @@
       <c r="N289" s="8"/>
       <c r="O289" s="8"/>
       <c r="P289" s="8"/>
-    </row>
-    <row r="290" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q289" s="8"/>
+      <c r="R289" s="8"/>
+    </row>
+    <row r="290" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A290" s="8">
         <v>285</v>
       </c>
@@ -13414,8 +13990,10 @@
       <c r="N290" s="8"/>
       <c r="O290" s="8"/>
       <c r="P290" s="8"/>
-    </row>
-    <row r="291" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q290" s="8"/>
+      <c r="R290" s="8"/>
+    </row>
+    <row r="291" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A291" s="8">
         <v>286</v>
       </c>
@@ -13454,8 +14032,10 @@
       <c r="N291" s="8"/>
       <c r="O291" s="8"/>
       <c r="P291" s="8"/>
-    </row>
-    <row r="292" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q291" s="8"/>
+      <c r="R291" s="8"/>
+    </row>
+    <row r="292" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A292" s="8">
         <v>287</v>
       </c>
@@ -13496,8 +14076,10 @@
       <c r="N292" s="8"/>
       <c r="O292" s="8"/>
       <c r="P292" s="8"/>
-    </row>
-    <row r="293" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q292" s="8"/>
+      <c r="R292" s="8"/>
+    </row>
+    <row r="293" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A293" s="8">
         <v>288</v>
       </c>
@@ -13536,8 +14118,10 @@
       <c r="N293" s="8"/>
       <c r="O293" s="8"/>
       <c r="P293" s="8"/>
-    </row>
-    <row r="294" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q293" s="8"/>
+      <c r="R293" s="8"/>
+    </row>
+    <row r="294" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A294" s="8">
         <v>289</v>
       </c>
@@ -13578,8 +14162,10 @@
       <c r="N294" s="8"/>
       <c r="O294" s="8"/>
       <c r="P294" s="8"/>
-    </row>
-    <row r="295" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q294" s="8"/>
+      <c r="R294" s="8"/>
+    </row>
+    <row r="295" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A295" s="10">
         <v>290</v>
       </c>
@@ -13622,8 +14208,10 @@
       </c>
       <c r="O295" s="10"/>
       <c r="P295" s="10"/>
-    </row>
-    <row r="296" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q295" s="10"/>
+      <c r="R295" s="10"/>
+    </row>
+    <row r="296" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A296" s="10">
         <v>291</v>
       </c>
@@ -13666,8 +14254,10 @@
       </c>
       <c r="O296" s="10"/>
       <c r="P296" s="10"/>
-    </row>
-    <row r="297" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q296" s="10"/>
+      <c r="R296" s="10"/>
+    </row>
+    <row r="297" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A297" s="10">
         <v>292</v>
       </c>
@@ -13710,8 +14300,10 @@
       </c>
       <c r="O297" s="10"/>
       <c r="P297" s="10"/>
-    </row>
-    <row r="298" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q297" s="10"/>
+      <c r="R297" s="10"/>
+    </row>
+    <row r="298" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A298" s="10">
         <v>293</v>
       </c>
@@ -13754,8 +14346,10 @@
       </c>
       <c r="O298" s="10"/>
       <c r="P298" s="10"/>
-    </row>
-    <row r="299" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q298" s="10"/>
+      <c r="R298" s="10"/>
+    </row>
+    <row r="299" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A299" s="10">
         <v>294</v>
       </c>
@@ -13798,8 +14392,10 @@
       </c>
       <c r="O299" s="10"/>
       <c r="P299" s="10"/>
-    </row>
-    <row r="300" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q299" s="10"/>
+      <c r="R299" s="10"/>
+    </row>
+    <row r="300" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A300" s="10">
         <v>295</v>
       </c>
@@ -13844,8 +14440,10 @@
       </c>
       <c r="O300" s="10"/>
       <c r="P300" s="10"/>
-    </row>
-    <row r="301" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q300" s="10"/>
+      <c r="R300" s="10"/>
+    </row>
+    <row r="301" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A301" s="10">
         <v>296</v>
       </c>
@@ -13890,8 +14488,10 @@
       </c>
       <c r="O301" s="10"/>
       <c r="P301" s="10"/>
-    </row>
-    <row r="302" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q301" s="10"/>
+      <c r="R301" s="10"/>
+    </row>
+    <row r="302" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A302" s="10">
         <v>297</v>
       </c>
@@ -13936,8 +14536,10 @@
       </c>
       <c r="O302" s="10"/>
       <c r="P302" s="10"/>
-    </row>
-    <row r="303" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q302" s="10"/>
+      <c r="R302" s="10"/>
+    </row>
+    <row r="303" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A303" s="10">
         <v>298</v>
       </c>
@@ -13980,8 +14582,10 @@
       </c>
       <c r="O303" s="10"/>
       <c r="P303" s="10"/>
-    </row>
-    <row r="304" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q303" s="10"/>
+      <c r="R303" s="10"/>
+    </row>
+    <row r="304" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A304" s="10">
         <v>299</v>
       </c>
@@ -14024,8 +14628,10 @@
       </c>
       <c r="O304" s="10"/>
       <c r="P304" s="10"/>
-    </row>
-    <row r="305" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q304" s="10"/>
+      <c r="R304" s="10"/>
+    </row>
+    <row r="305" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A305" s="10">
         <v>300</v>
       </c>
@@ -14070,8 +14676,10 @@
       </c>
       <c r="O305" s="10"/>
       <c r="P305" s="10"/>
-    </row>
-    <row r="306" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q305" s="10"/>
+      <c r="R305" s="10"/>
+    </row>
+    <row r="306" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A306" s="10">
         <v>301</v>
       </c>
@@ -14116,8 +14724,10 @@
       </c>
       <c r="O306" s="10"/>
       <c r="P306" s="10"/>
-    </row>
-    <row r="307" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q306" s="10"/>
+      <c r="R306" s="10"/>
+    </row>
+    <row r="307" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A307" s="10">
         <v>302</v>
       </c>
@@ -14160,8 +14770,10 @@
       </c>
       <c r="O307" s="10"/>
       <c r="P307" s="10"/>
-    </row>
-    <row r="308" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q307" s="10"/>
+      <c r="R307" s="10"/>
+    </row>
+    <row r="308" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A308" s="10">
         <v>303</v>
       </c>
@@ -14204,8 +14816,10 @@
       </c>
       <c r="O308" s="10"/>
       <c r="P308" s="10"/>
-    </row>
-    <row r="309" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q308" s="10"/>
+      <c r="R308" s="10"/>
+    </row>
+    <row r="309" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A309" s="10">
         <v>304</v>
       </c>
@@ -14250,8 +14864,10 @@
       </c>
       <c r="O309" s="10"/>
       <c r="P309" s="10"/>
-    </row>
-    <row r="310" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q309" s="10"/>
+      <c r="R309" s="10"/>
+    </row>
+    <row r="310" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A310" s="10">
         <v>305</v>
       </c>
@@ -14296,8 +14912,10 @@
       </c>
       <c r="O310" s="10"/>
       <c r="P310" s="10"/>
-    </row>
-    <row r="311" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q310" s="10"/>
+      <c r="R310" s="10"/>
+    </row>
+    <row r="311" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A311" s="10">
         <v>306</v>
       </c>
@@ -14340,8 +14958,10 @@
       </c>
       <c r="O311" s="10"/>
       <c r="P311" s="10"/>
-    </row>
-    <row r="312" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q311" s="10"/>
+      <c r="R311" s="10"/>
+    </row>
+    <row r="312" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A312" s="10">
         <v>307</v>
       </c>
@@ -14384,8 +15004,10 @@
       </c>
       <c r="O312" s="10"/>
       <c r="P312" s="10"/>
-    </row>
-    <row r="313" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q312" s="10"/>
+      <c r="R312" s="10"/>
+    </row>
+    <row r="313" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A313" s="10">
         <v>308</v>
       </c>
@@ -14428,8 +15050,10 @@
       </c>
       <c r="O313" s="10"/>
       <c r="P313" s="10"/>
-    </row>
-    <row r="314" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="Q313" s="10"/>
+      <c r="R313" s="10"/>
+    </row>
+    <row r="314" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A314" s="10">
         <v>309</v>
       </c>
@@ -14474,8 +15098,10 @@
       </c>
       <c r="O314" s="10"/>
       <c r="P314" s="10"/>
-    </row>
-    <row r="315" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q314" s="10"/>
+      <c r="R314" s="10"/>
+    </row>
+    <row r="315" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A315" s="10">
         <v>310</v>
       </c>
@@ -14520,8 +15146,10 @@
       </c>
       <c r="O315" s="10"/>
       <c r="P315" s="10"/>
-    </row>
-    <row r="316" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q315" s="10"/>
+      <c r="R315" s="10"/>
+    </row>
+    <row r="316" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A316" s="10">
         <v>311</v>
       </c>
@@ -14564,8 +15192,10 @@
       </c>
       <c r="O316" s="10"/>
       <c r="P316" s="10"/>
-    </row>
-    <row r="317" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q316" s="10"/>
+      <c r="R316" s="10"/>
+    </row>
+    <row r="317" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A317" s="10">
         <v>312</v>
       </c>
@@ -14608,8 +15238,10 @@
       </c>
       <c r="O317" s="10"/>
       <c r="P317" s="10"/>
-    </row>
-    <row r="318" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q317" s="10"/>
+      <c r="R317" s="10"/>
+    </row>
+    <row r="318" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A318" s="10">
         <v>313</v>
       </c>
@@ -14652,8 +15284,10 @@
       </c>
       <c r="O318" s="10"/>
       <c r="P318" s="10"/>
-    </row>
-    <row r="319" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q318" s="10"/>
+      <c r="R318" s="10"/>
+    </row>
+    <row r="319" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A319" s="10">
         <v>314</v>
       </c>
@@ -14696,8 +15330,10 @@
       </c>
       <c r="O319" s="10"/>
       <c r="P319" s="10"/>
-    </row>
-    <row r="320" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q319" s="10"/>
+      <c r="R319" s="10"/>
+    </row>
+    <row r="320" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A320" s="10">
         <v>315</v>
       </c>
@@ -14740,8 +15376,10 @@
       </c>
       <c r="O320" s="10"/>
       <c r="P320" s="10"/>
-    </row>
-    <row r="321" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q320" s="10"/>
+      <c r="R320" s="10"/>
+    </row>
+    <row r="321" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A321" s="10">
         <v>316</v>
       </c>
@@ -14784,8 +15422,10 @@
       </c>
       <c r="O321" s="10"/>
       <c r="P321" s="10"/>
-    </row>
-    <row r="322" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q321" s="10"/>
+      <c r="R321" s="10"/>
+    </row>
+    <row r="322" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A322" s="10">
         <v>317</v>
       </c>
@@ -14828,8 +15468,10 @@
       </c>
       <c r="O322" s="10"/>
       <c r="P322" s="10"/>
-    </row>
-    <row r="323" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q322" s="10"/>
+      <c r="R322" s="10"/>
+    </row>
+    <row r="323" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A323" s="10">
         <v>318</v>
       </c>
@@ -14872,8 +15514,10 @@
       </c>
       <c r="O323" s="10"/>
       <c r="P323" s="10"/>
-    </row>
-    <row r="324" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q323" s="10"/>
+      <c r="R323" s="10"/>
+    </row>
+    <row r="324" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A324" s="10">
         <v>319</v>
       </c>
@@ -14916,8 +15560,10 @@
       </c>
       <c r="O324" s="10"/>
       <c r="P324" s="10"/>
-    </row>
-    <row r="325" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q324" s="10"/>
+      <c r="R324" s="10"/>
+    </row>
+    <row r="325" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A325" s="10">
         <v>320</v>
       </c>
@@ -14960,8 +15606,10 @@
       </c>
       <c r="O325" s="10"/>
       <c r="P325" s="10"/>
-    </row>
-    <row r="326" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q325" s="10"/>
+      <c r="R325" s="10"/>
+    </row>
+    <row r="326" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A326" s="10">
         <v>321</v>
       </c>
@@ -15004,8 +15652,10 @@
       </c>
       <c r="O326" s="10"/>
       <c r="P326" s="10"/>
-    </row>
-    <row r="327" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q326" s="10"/>
+      <c r="R326" s="10"/>
+    </row>
+    <row r="327" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A327" s="10">
         <v>322</v>
       </c>
@@ -15048,8 +15698,10 @@
       </c>
       <c r="O327" s="10"/>
       <c r="P327" s="10"/>
-    </row>
-    <row r="328" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q327" s="10"/>
+      <c r="R327" s="10"/>
+    </row>
+    <row r="328" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A328" s="10">
         <v>323</v>
       </c>
@@ -15092,8 +15744,10 @@
       </c>
       <c r="O328" s="10"/>
       <c r="P328" s="10"/>
-    </row>
-    <row r="329" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q328" s="10"/>
+      <c r="R328" s="10"/>
+    </row>
+    <row r="329" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A329" s="10">
         <v>324</v>
       </c>
@@ -15138,8 +15792,10 @@
       </c>
       <c r="O329" s="10"/>
       <c r="P329" s="10"/>
-    </row>
-    <row r="330" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q329" s="10"/>
+      <c r="R329" s="10"/>
+    </row>
+    <row r="330" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A330" s="10">
         <v>325</v>
       </c>
@@ -15184,8 +15840,10 @@
       </c>
       <c r="O330" s="10"/>
       <c r="P330" s="10"/>
-    </row>
-    <row r="331" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q330" s="10"/>
+      <c r="R330" s="10"/>
+    </row>
+    <row r="331" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A331" s="10">
         <v>326</v>
       </c>
@@ -15230,8 +15888,10 @@
       </c>
       <c r="O331" s="10"/>
       <c r="P331" s="10"/>
-    </row>
-    <row r="332" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q331" s="10"/>
+      <c r="R331" s="10"/>
+    </row>
+    <row r="332" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A332" s="10">
         <v>327</v>
       </c>
@@ -15276,8 +15936,10 @@
       </c>
       <c r="O332" s="10"/>
       <c r="P332" s="10"/>
-    </row>
-    <row r="333" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q332" s="10"/>
+      <c r="R332" s="10"/>
+    </row>
+    <row r="333" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A333" s="10">
         <v>328</v>
       </c>
@@ -15320,8 +15982,10 @@
       </c>
       <c r="O333" s="10"/>
       <c r="P333" s="10"/>
-    </row>
-    <row r="334" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q333" s="10"/>
+      <c r="R333" s="10"/>
+    </row>
+    <row r="334" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A334" s="10">
         <v>329</v>
       </c>
@@ -15364,8 +16028,10 @@
       </c>
       <c r="O334" s="10"/>
       <c r="P334" s="10"/>
-    </row>
-    <row r="335" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q334" s="10"/>
+      <c r="R334" s="10"/>
+    </row>
+    <row r="335" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A335" s="10">
         <v>330</v>
       </c>
@@ -15410,8 +16076,10 @@
       </c>
       <c r="O335" s="10"/>
       <c r="P335" s="10"/>
-    </row>
-    <row r="336" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q335" s="10"/>
+      <c r="R335" s="10"/>
+    </row>
+    <row r="336" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A336" s="10">
         <v>331</v>
       </c>
@@ -15456,8 +16124,10 @@
       </c>
       <c r="O336" s="10"/>
       <c r="P336" s="10"/>
-    </row>
-    <row r="337" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q336" s="10"/>
+      <c r="R336" s="10"/>
+    </row>
+    <row r="337" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A337" s="10">
         <v>332</v>
       </c>
@@ -15502,8 +16172,10 @@
       </c>
       <c r="O337" s="10"/>
       <c r="P337" s="10"/>
-    </row>
-    <row r="338" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q337" s="10"/>
+      <c r="R337" s="10"/>
+    </row>
+    <row r="338" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A338" s="10">
         <v>333</v>
       </c>
@@ -15548,8 +16220,10 @@
       </c>
       <c r="O338" s="10"/>
       <c r="P338" s="10"/>
-    </row>
-    <row r="339" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q338" s="10"/>
+      <c r="R338" s="10"/>
+    </row>
+    <row r="339" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A339" s="10">
         <v>334</v>
       </c>
@@ -15592,8 +16266,10 @@
       </c>
       <c r="O339" s="10"/>
       <c r="P339" s="10"/>
-    </row>
-    <row r="340" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q339" s="10"/>
+      <c r="R339" s="10"/>
+    </row>
+    <row r="340" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A340" s="10">
         <v>335</v>
       </c>
@@ -15636,8 +16312,10 @@
       </c>
       <c r="O340" s="10"/>
       <c r="P340" s="10"/>
-    </row>
-    <row r="341" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q340" s="10"/>
+      <c r="R340" s="10"/>
+    </row>
+    <row r="341" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A341" s="10">
         <v>336</v>
       </c>
@@ -15680,8 +16358,10 @@
       </c>
       <c r="O341" s="10"/>
       <c r="P341" s="10"/>
-    </row>
-    <row r="342" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q341" s="10"/>
+      <c r="R341" s="10"/>
+    </row>
+    <row r="342" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A342" s="10">
         <v>337</v>
       </c>
@@ -15724,8 +16404,10 @@
       </c>
       <c r="O342" s="10"/>
       <c r="P342" s="10"/>
-    </row>
-    <row r="343" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q342" s="10"/>
+      <c r="R342" s="10"/>
+    </row>
+    <row r="343" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A343" s="10">
         <v>338</v>
       </c>
@@ -15768,8 +16450,10 @@
       </c>
       <c r="O343" s="10"/>
       <c r="P343" s="10"/>
-    </row>
-    <row r="344" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q343" s="10"/>
+      <c r="R343" s="10"/>
+    </row>
+    <row r="344" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A344" s="10">
         <v>339</v>
       </c>
@@ -15812,8 +16496,10 @@
       </c>
       <c r="O344" s="10"/>
       <c r="P344" s="10"/>
-    </row>
-    <row r="345" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q344" s="10"/>
+      <c r="R344" s="10"/>
+    </row>
+    <row r="345" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A345" s="10">
         <v>340</v>
       </c>
@@ -15858,8 +16544,10 @@
       </c>
       <c r="O345" s="10"/>
       <c r="P345" s="10"/>
-    </row>
-    <row r="346" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q345" s="10"/>
+      <c r="R345" s="10"/>
+    </row>
+    <row r="346" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A346" s="10">
         <v>341</v>
       </c>
@@ -15904,8 +16592,10 @@
       </c>
       <c r="O346" s="10"/>
       <c r="P346" s="10"/>
-    </row>
-    <row r="347" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q346" s="10"/>
+      <c r="R346" s="10"/>
+    </row>
+    <row r="347" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A347" s="10">
         <v>342</v>
       </c>
@@ -15950,8 +16640,10 @@
       </c>
       <c r="O347" s="10"/>
       <c r="P347" s="10"/>
-    </row>
-    <row r="348" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q347" s="10"/>
+      <c r="R347" s="10"/>
+    </row>
+    <row r="348" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A348" s="10">
         <v>343</v>
       </c>
@@ -15994,8 +16686,10 @@
       </c>
       <c r="O348" s="10"/>
       <c r="P348" s="10"/>
-    </row>
-    <row r="349" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q348" s="10"/>
+      <c r="R348" s="10"/>
+    </row>
+    <row r="349" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A349" s="15">
         <v>344</v>
       </c>
@@ -16038,8 +16732,10 @@
       <c r="N349" s="15"/>
       <c r="O349" s="15"/>
       <c r="P349" s="15"/>
-    </row>
-    <row r="350" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q349" s="15"/>
+      <c r="R349" s="15"/>
+    </row>
+    <row r="350" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A350" s="15">
         <v>345</v>
       </c>
@@ -16082,8 +16778,10 @@
       <c r="N350" s="15"/>
       <c r="O350" s="15"/>
       <c r="P350" s="15"/>
-    </row>
-    <row r="351" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q350" s="15"/>
+      <c r="R350" s="15"/>
+    </row>
+    <row r="351" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A351" s="15">
         <v>346</v>
       </c>
@@ -16126,8 +16824,10 @@
       <c r="N351" s="15"/>
       <c r="O351" s="15"/>
       <c r="P351" s="15"/>
-    </row>
-    <row r="352" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q351" s="15"/>
+      <c r="R351" s="15"/>
+    </row>
+    <row r="352" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A352" s="15">
         <v>347</v>
       </c>
@@ -16170,6 +16870,8 @@
       <c r="N352" s="15"/>
       <c r="O352" s="15"/>
       <c r="P352" s="15"/>
+      <c r="Q352" s="15"/>
+      <c r="R352" s="15"/>
     </row>
     <row r="357" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F357" s="18"/>

</xml_diff>